<commit_message>
📊 Update NAIC content history - 2026-02-24
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40C5F77-DC61-4729-AC29-54E7D389E37E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4EAA2C-B6E0-4FA9-BBF8-3F838C11E86A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -2913,51 +2913,51 @@
           <cell r="H56">
             <v>46074</v>
           </cell>
-          <cell r="I56" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J56" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K56" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L56" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I56">
+            <v>3.8600000000000002E-2</v>
+          </cell>
+          <cell r="J56">
+            <v>4.2000000000000003E-2</v>
+          </cell>
+          <cell r="K56">
+            <v>4.4699999999999997E-2</v>
+          </cell>
+          <cell r="L56">
+            <v>4.7399999999999998E-2</v>
           </cell>
         </row>
         <row r="57">
           <cell r="H57">
             <v>46075</v>
           </cell>
-          <cell r="I57" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J57" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K57" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L57" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I57">
+            <v>3.8600000000000002E-2</v>
+          </cell>
+          <cell r="J57">
+            <v>4.2000000000000003E-2</v>
+          </cell>
+          <cell r="K57">
+            <v>4.4699999999999997E-2</v>
+          </cell>
+          <cell r="L57">
+            <v>4.7399999999999998E-2</v>
           </cell>
         </row>
         <row r="58">
           <cell r="H58">
             <v>46076</v>
           </cell>
-          <cell r="I58" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J58" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K58" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L58" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I58">
+            <v>3.8600000000000002E-2</v>
+          </cell>
+          <cell r="J58">
+            <v>4.2000000000000003E-2</v>
+          </cell>
+          <cell r="K58">
+            <v>4.4699999999999997E-2</v>
+          </cell>
+          <cell r="L58">
+            <v>4.7399999999999998E-2</v>
           </cell>
         </row>
         <row r="59">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,26 +8346,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8398,26 +8381,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8593,16 +8559,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8611,7 +8577,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8620,7 +8586,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8637,7 +8603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8659,7 +8625,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8681,7 +8647,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8703,7 +8669,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8725,7 +8691,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8747,7 +8713,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8769,7 +8735,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8791,7 +8757,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8813,7 +8779,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8835,7 +8801,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8857,7 +8823,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8879,7 +8845,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8901,7 +8867,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8923,7 +8889,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8945,7 +8911,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8967,7 +8933,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8989,7 +8955,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -9011,7 +8977,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9033,7 +8999,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9055,7 +9021,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9077,7 +9043,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9099,7 +9065,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9121,7 +9087,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9143,7 +9109,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9165,7 +9131,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9187,7 +9153,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9209,7 +9175,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9231,7 +9197,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9253,7 +9219,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9275,7 +9241,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9297,7 +9263,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9319,7 +9285,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9341,7 +9307,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9363,7 +9329,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9385,7 +9351,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9407,7 +9373,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9429,7 +9395,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9451,7 +9417,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9473,7 +9439,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9495,7 +9461,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9517,7 +9483,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9539,7 +9505,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9561,7 +9527,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9583,7 +9549,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9605,7 +9571,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9627,7 +9593,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9649,7 +9615,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9671,7 +9637,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9693,7 +9659,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9715,7 +9681,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9737,7 +9703,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9759,73 +9725,73 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
       </c>
-      <c r="B55" s="17" t="str">
+      <c r="B55" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I56</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C55" s="47" t="str">
+        <v>3.8600000000000002E-2</v>
+      </c>
+      <c r="C55" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J56</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D55" s="47" t="str">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="D55" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K56</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E55" s="5" t="str">
+        <v>4.4699999999999997E-2</v>
+      </c>
+      <c r="E55" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L56</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.7399999999999998E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
       </c>
-      <c r="B56" s="17" t="str">
+      <c r="B56" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I57</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C56" s="47" t="str">
+        <v>3.8600000000000002E-2</v>
+      </c>
+      <c r="C56" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J57</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D56" s="47" t="str">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="D56" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K57</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E56" s="5" t="str">
+        <v>4.4699999999999997E-2</v>
+      </c>
+      <c r="E56" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L57</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.7399999999999998E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
       </c>
-      <c r="B57" s="17" t="str">
+      <c r="B57" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I58</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C57" s="47" t="str">
+        <v>3.8600000000000002E-2</v>
+      </c>
+      <c r="C57" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J58</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D57" s="47" t="str">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="D57" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K58</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E57" s="5" t="str">
+        <v>4.4699999999999997E-2</v>
+      </c>
+      <c r="E57" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L58</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.7399999999999998E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9847,7 +9813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9869,7 +9835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9891,7 +9857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9913,7 +9879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9935,7 +9901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9957,7 +9923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9979,7 +9945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -10001,7 +9967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10023,7 +9989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10045,7 +10011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10067,7 +10033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10089,7 +10055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10111,7 +10077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10133,7 +10099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10155,7 +10121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10177,7 +10143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10199,7 +10165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10221,7 +10187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10243,7 +10209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10265,7 +10231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10287,7 +10253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10309,7 +10275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10331,7 +10297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10353,7 +10319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10375,7 +10341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10397,7 +10363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10419,7 +10385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10441,7 +10407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10463,7 +10429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10485,7 +10451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10507,7 +10473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10529,7 +10495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10551,7 +10517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10573,7 +10539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10595,7 +10561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10617,7 +10583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10639,7 +10605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10661,7 +10627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10683,7 +10649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10705,7 +10671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10727,7 +10693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10749,7 +10715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10771,7 +10737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10793,7 +10759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10815,7 +10781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10837,7 +10803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10859,7 +10825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10881,7 +10847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10903,7 +10869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10925,7 +10891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10947,7 +10913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10969,7 +10935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10991,7 +10957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -11013,7 +10979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11035,7 +11001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11057,7 +11023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11079,7 +11045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11101,7 +11067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11123,7 +11089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11145,7 +11111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11167,7 +11133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11189,7 +11155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11211,7 +11177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11233,7 +11199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11255,7 +11221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11277,7 +11243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11299,7 +11265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11321,7 +11287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11343,7 +11309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11365,7 +11331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11387,7 +11353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11409,7 +11375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11431,7 +11397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11453,7 +11419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11475,7 +11441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11497,7 +11463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11519,7 +11485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11541,7 +11507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11563,7 +11529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11585,7 +11551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11607,7 +11573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11629,7 +11595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11651,7 +11617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11673,7 +11639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11695,7 +11661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11717,7 +11683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11739,7 +11705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11761,7 +11727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11783,7 +11749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11805,7 +11771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11827,7 +11793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11849,7 +11815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11871,7 +11837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11893,7 +11859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11915,7 +11881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11937,7 +11903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11959,7 +11925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11981,7 +11947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -12003,7 +11969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12025,7 +11991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12047,7 +12013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12069,7 +12035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12091,7 +12057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12113,7 +12079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12135,7 +12101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12157,7 +12123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12179,7 +12145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12201,7 +12167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12223,7 +12189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12245,7 +12211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12267,7 +12233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12289,7 +12255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12311,7 +12277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12333,7 +12299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12355,7 +12321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12377,7 +12343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12399,7 +12365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12421,7 +12387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12443,7 +12409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12465,7 +12431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12487,7 +12453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12509,7 +12475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12531,7 +12497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12553,7 +12519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12575,7 +12541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12597,7 +12563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12619,7 +12585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12641,7 +12607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12663,7 +12629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12685,7 +12651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12707,7 +12673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12729,7 +12695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12751,7 +12717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12773,7 +12739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12795,7 +12761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12817,7 +12783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12839,7 +12805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12861,7 +12827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12883,7 +12849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12905,7 +12871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12927,7 +12893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12949,7 +12915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12971,7 +12937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12993,7 +12959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13015,7 +12981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13037,7 +13003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13059,7 +13025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13081,7 +13047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13103,7 +13069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13125,7 +13091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13147,7 +13113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13169,7 +13135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13191,7 +13157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13213,7 +13179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13235,7 +13201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13257,7 +13223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13279,7 +13245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13301,7 +13267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13323,7 +13289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13345,7 +13311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13367,7 +13333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13389,7 +13355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13411,7 +13377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13433,7 +13399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13455,7 +13421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13477,7 +13443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13499,7 +13465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13521,7 +13487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13543,7 +13509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13565,7 +13531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13587,7 +13553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13609,7 +13575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13631,7 +13597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13653,7 +13619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13675,7 +13641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13697,7 +13663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13719,7 +13685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13741,7 +13707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13763,7 +13729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13785,7 +13751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13807,7 +13773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13829,7 +13795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13851,7 +13817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13873,7 +13839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13895,7 +13861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13917,7 +13883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13939,7 +13905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13961,7 +13927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13983,7 +13949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -14005,7 +13971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14027,7 +13993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14049,7 +14015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14071,7 +14037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14093,7 +14059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14115,7 +14081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14137,7 +14103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14159,7 +14125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14181,7 +14147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14203,7 +14169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14225,7 +14191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14247,7 +14213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14269,7 +14235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14291,7 +14257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14313,7 +14279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14335,7 +14301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14357,7 +14323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14379,7 +14345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14401,7 +14367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14423,7 +14389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14445,7 +14411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14467,7 +14433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14489,7 +14455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14511,7 +14477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14533,7 +14499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14555,7 +14521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14577,7 +14543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14599,7 +14565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14621,7 +14587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14643,7 +14609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14665,7 +14631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14687,7 +14653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14709,7 +14675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14731,7 +14697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14753,7 +14719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14775,7 +14741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14797,7 +14763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14819,7 +14785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14841,7 +14807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14863,7 +14829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14885,7 +14851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14907,7 +14873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14929,7 +14895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14951,7 +14917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14973,7 +14939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14995,7 +14961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15017,7 +14983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15039,7 +15005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15061,7 +15027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15083,7 +15049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15105,7 +15071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15127,7 +15093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15149,7 +15115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15171,7 +15137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15193,7 +15159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15215,7 +15181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15237,7 +15203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15259,7 +15225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15281,7 +15247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15303,7 +15269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15325,7 +15291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15347,7 +15313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15369,7 +15335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15391,7 +15357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15413,7 +15379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15435,7 +15401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15457,7 +15423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15479,7 +15445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15501,7 +15467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15523,7 +15489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15545,7 +15511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15567,7 +15533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15589,7 +15555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15611,7 +15577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15633,7 +15599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15655,7 +15621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15677,7 +15643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15699,7 +15665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15721,7 +15687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15743,7 +15709,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15765,7 +15731,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15787,7 +15753,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15809,7 +15775,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15831,7 +15797,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15853,7 +15819,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15875,7 +15841,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15897,7 +15863,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15919,7 +15885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15941,7 +15907,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15963,7 +15929,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15985,7 +15951,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -16007,7 +15973,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16029,7 +15995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16051,7 +16017,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16073,7 +16039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16095,7 +16061,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16117,7 +16083,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16139,7 +16105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16161,7 +16127,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16183,7 +16149,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16205,7 +16171,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16227,7 +16193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16249,7 +16215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16271,7 +16237,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16293,7 +16259,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16315,7 +16281,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16337,7 +16303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16359,7 +16325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16381,7 +16347,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16403,7 +16369,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16425,7 +16391,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16447,7 +16413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16469,7 +16435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16491,7 +16457,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16513,7 +16479,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16535,7 +16501,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16557,7 +16523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16579,7 +16545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16601,7 +16567,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16623,7 +16589,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16645,7 +16611,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16667,7 +16633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16689,37 +16655,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16735,13 +16701,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16750,14 +16716,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16766,7 +16732,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16775,7 +16741,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16792,7 +16758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16814,7 +16780,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16836,7 +16802,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16858,7 +16824,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16880,7 +16846,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16897,13 +16863,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16912,7 +16878,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16921,12 +16887,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16935,7 +16901,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16952,7 +16918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16976,7 +16942,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -17000,7 +16966,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17024,7 +16990,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17048,7 +17014,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17056,7 +17022,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17064,7 +17030,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17074,7 +17040,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17084,7 +17050,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17102,7 +17068,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17124,7 +17090,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17146,7 +17112,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17168,7 +17134,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17190,7 +17156,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17198,7 +17164,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17206,7 +17172,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17216,7 +17182,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17226,7 +17192,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17242,7 +17208,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17262,7 +17228,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17282,7 +17248,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17302,7 +17268,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17322,7 +17288,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17331,7 +17297,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17342,7 +17308,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17353,7 +17319,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17376,7 +17342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17411,7 +17377,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17446,7 +17412,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17481,7 +17447,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17533,193 +17499,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17889,7 +17855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18023,7 +17989,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18197,7 +18163,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18371,7 +18337,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18545,7 +18511,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18719,7 +18685,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18893,7 +18859,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19067,7 +19033,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19241,7 +19207,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19415,7 +19381,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19589,7 +19555,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19763,7 +19729,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19937,7 +19903,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20111,7 +20077,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20285,7 +20251,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20459,7 +20425,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20633,7 +20599,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20807,7 +20773,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20981,7 +20947,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21155,7 +21121,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21329,7 +21295,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21503,7 +21469,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21677,7 +21643,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21851,7 +21817,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22025,7 +21991,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22199,7 +22165,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22373,7 +22339,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22547,7 +22513,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22721,7 +22687,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22895,7 +22861,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23069,7 +23035,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23243,7 +23209,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23419,18 +23385,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23443,7 +23409,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23464,7 +23430,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-02-25
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4EAA2C-B6E0-4FA9-BBF8-3F838C11E86A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D0EA38-9ECF-4570-9F91-4D0BF44696CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -2964,17 +2964,17 @@
           <cell r="H59">
             <v>46077</v>
           </cell>
-          <cell r="I59" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J59" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K59" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L59" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I59">
+            <v>3.8300000000000001E-2</v>
+          </cell>
+          <cell r="J59">
+            <v>4.1700000000000001E-2</v>
+          </cell>
+          <cell r="K59">
+            <v>4.4400000000000002E-2</v>
+          </cell>
+          <cell r="L59">
+            <v>4.7300000000000002E-2</v>
           </cell>
         </row>
         <row r="60">
@@ -8559,16 +8559,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8577,7 +8577,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8586,7 +8586,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8603,7 +8603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8625,7 +8625,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8647,7 +8647,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8669,7 +8669,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8691,7 +8691,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8713,7 +8713,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8735,7 +8735,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8757,7 +8757,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8779,7 +8779,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8801,7 +8801,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8823,7 +8823,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8845,7 +8845,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8867,7 +8867,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8889,7 +8889,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8911,7 +8911,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8933,7 +8933,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8955,7 +8955,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8977,7 +8977,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -8999,7 +8999,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9021,7 +9021,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9043,7 +9043,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9065,7 +9065,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9087,7 +9087,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9109,7 +9109,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9131,7 +9131,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9153,7 +9153,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9175,7 +9175,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9197,7 +9197,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9219,7 +9219,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9241,7 +9241,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9263,7 +9263,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9285,7 +9285,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9307,7 +9307,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9329,7 +9329,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9351,7 +9351,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9373,7 +9373,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9395,7 +9395,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9417,7 +9417,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9439,7 +9439,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9461,7 +9461,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9483,7 +9483,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9505,7 +9505,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9527,7 +9527,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9549,7 +9549,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9571,7 +9571,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9593,7 +9593,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9615,7 +9615,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9637,7 +9637,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9659,7 +9659,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9681,7 +9681,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9703,7 +9703,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9725,7 +9725,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9747,7 +9747,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9769,7 +9769,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9791,29 +9791,29 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
       </c>
-      <c r="B58" s="17" t="str">
+      <c r="B58" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I59</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C58" s="47" t="str">
+        <v>3.8300000000000001E-2</v>
+      </c>
+      <c r="C58" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J59</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D58" s="47" t="str">
+        <v>4.1700000000000001E-2</v>
+      </c>
+      <c r="D58" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K59</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E58" s="5" t="str">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="E58" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L59</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4.7300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9835,7 +9835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9857,7 +9857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9879,7 +9879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9901,7 +9901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9923,7 +9923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9945,7 +9945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9967,7 +9967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -9989,7 +9989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10011,7 +10011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10033,7 +10033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10055,7 +10055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10077,7 +10077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10099,7 +10099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10121,7 +10121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10143,7 +10143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10165,7 +10165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10187,7 +10187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10209,7 +10209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10231,7 +10231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10253,7 +10253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10275,7 +10275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10297,7 +10297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10319,7 +10319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10341,7 +10341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10363,7 +10363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10385,7 +10385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10407,7 +10407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10429,7 +10429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10451,7 +10451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10473,7 +10473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10495,7 +10495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10517,7 +10517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10539,7 +10539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10561,7 +10561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10583,7 +10583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10605,7 +10605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10627,7 +10627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10649,7 +10649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10671,7 +10671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10693,7 +10693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10715,7 +10715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10737,7 +10737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10759,7 +10759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10781,7 +10781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10803,7 +10803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10825,7 +10825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10847,7 +10847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10869,7 +10869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10891,7 +10891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10913,7 +10913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10935,7 +10935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10957,7 +10957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10979,7 +10979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11001,7 +11001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11023,7 +11023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11045,7 +11045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11067,7 +11067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11089,7 +11089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11111,7 +11111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11133,7 +11133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11155,7 +11155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11177,7 +11177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11199,7 +11199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11221,7 +11221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11243,7 +11243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11265,7 +11265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11287,7 +11287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11309,7 +11309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11331,7 +11331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11353,7 +11353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11375,7 +11375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11397,7 +11397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11419,7 +11419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11441,7 +11441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11463,7 +11463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11485,7 +11485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11507,7 +11507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11529,7 +11529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11551,7 +11551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11573,7 +11573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11595,7 +11595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11617,7 +11617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11639,7 +11639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11661,7 +11661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11683,7 +11683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11705,7 +11705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11727,7 +11727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11749,7 +11749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11771,7 +11771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11793,7 +11793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11815,7 +11815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11837,7 +11837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11859,7 +11859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11881,7 +11881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11903,7 +11903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11925,7 +11925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11947,7 +11947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11969,7 +11969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -11991,7 +11991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12013,7 +12013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12035,7 +12035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12057,7 +12057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12079,7 +12079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12101,7 +12101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12123,7 +12123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12145,7 +12145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12167,7 +12167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12189,7 +12189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12211,7 +12211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12233,7 +12233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12255,7 +12255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12277,7 +12277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12299,7 +12299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12321,7 +12321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12343,7 +12343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12365,7 +12365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12387,7 +12387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12409,7 +12409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12431,7 +12431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12453,7 +12453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12475,7 +12475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12497,7 +12497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12519,7 +12519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12541,7 +12541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12563,7 +12563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12585,7 +12585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12607,7 +12607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12629,7 +12629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12651,7 +12651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12673,7 +12673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12695,7 +12695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12717,7 +12717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12739,7 +12739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12761,7 +12761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12783,7 +12783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12805,7 +12805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12827,7 +12827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12849,7 +12849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12871,7 +12871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12893,7 +12893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12915,7 +12915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12937,7 +12937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12959,7 +12959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -12981,7 +12981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13003,7 +13003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13025,7 +13025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13047,7 +13047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13069,7 +13069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13091,7 +13091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13113,7 +13113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13135,7 +13135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13157,7 +13157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13179,7 +13179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13201,7 +13201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13223,7 +13223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13245,7 +13245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13267,7 +13267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13289,7 +13289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13311,7 +13311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13333,7 +13333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13355,7 +13355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13377,7 +13377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13399,7 +13399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13421,7 +13421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13443,7 +13443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13465,7 +13465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13487,7 +13487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13509,7 +13509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13531,7 +13531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13553,7 +13553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13575,7 +13575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13597,7 +13597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13619,7 +13619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13641,7 +13641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13663,7 +13663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13685,7 +13685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13707,7 +13707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13729,7 +13729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13751,7 +13751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13773,7 +13773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13795,7 +13795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13817,7 +13817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13839,7 +13839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13861,7 +13861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13883,7 +13883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13905,7 +13905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13927,7 +13927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13949,7 +13949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13971,7 +13971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -13993,7 +13993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14015,7 +14015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14037,7 +14037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14059,7 +14059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14081,7 +14081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14103,7 +14103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14125,7 +14125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14147,7 +14147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14169,7 +14169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14191,7 +14191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14213,7 +14213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14235,7 +14235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14257,7 +14257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14279,7 +14279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14301,7 +14301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14323,7 +14323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14345,7 +14345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14367,7 +14367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14389,7 +14389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14411,7 +14411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14433,7 +14433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14455,7 +14455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14477,7 +14477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14499,7 +14499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14521,7 +14521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14543,7 +14543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14565,7 +14565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14587,7 +14587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14609,7 +14609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14631,7 +14631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14653,7 +14653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14675,7 +14675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14697,7 +14697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14719,7 +14719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14741,7 +14741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14763,7 +14763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14785,7 +14785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14807,7 +14807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14829,7 +14829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14851,7 +14851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14873,7 +14873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14895,7 +14895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14917,7 +14917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14939,7 +14939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14961,7 +14961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -14983,7 +14983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15005,7 +15005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15027,7 +15027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15049,7 +15049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15071,7 +15071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15093,7 +15093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15115,7 +15115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15137,7 +15137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15159,7 +15159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15181,7 +15181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15203,7 +15203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15225,7 +15225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15247,7 +15247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15269,7 +15269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15291,7 +15291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15313,7 +15313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15335,7 +15335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15357,7 +15357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15379,7 +15379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15401,7 +15401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15423,7 +15423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15445,7 +15445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15467,7 +15467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15489,7 +15489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15511,7 +15511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15533,7 +15533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15555,7 +15555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15577,7 +15577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15599,7 +15599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15621,7 +15621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15643,7 +15643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15665,7 +15665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15687,7 +15687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15709,7 +15709,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15731,7 +15731,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15753,7 +15753,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15775,7 +15775,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15797,7 +15797,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15819,7 +15819,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15841,7 +15841,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15863,7 +15863,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15885,7 +15885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15907,7 +15907,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15929,7 +15929,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15951,7 +15951,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15973,7 +15973,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -15995,7 +15995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16017,7 +16017,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16039,7 +16039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16061,7 +16061,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16083,7 +16083,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16105,7 +16105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16127,7 +16127,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16149,7 +16149,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16171,7 +16171,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16193,7 +16193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16215,7 +16215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16237,7 +16237,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16259,7 +16259,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16281,7 +16281,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16303,7 +16303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16325,7 +16325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16347,7 +16347,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16369,7 +16369,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16391,7 +16391,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16413,7 +16413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16435,7 +16435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16457,7 +16457,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16479,7 +16479,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16501,7 +16501,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16523,7 +16523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16545,7 +16545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16567,7 +16567,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16589,7 +16589,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16611,7 +16611,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16633,7 +16633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16655,37 +16655,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16701,13 +16701,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16716,14 +16716,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16732,7 +16732,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16741,7 +16741,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16758,7 +16758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16780,7 +16780,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16802,7 +16802,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16824,7 +16824,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16846,7 +16846,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16863,13 +16863,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16878,7 +16878,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16887,12 +16887,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16901,7 +16901,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16918,7 +16918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16942,7 +16942,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16966,7 +16966,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -16990,7 +16990,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17014,7 +17014,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17022,7 +17022,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17030,7 +17030,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17040,7 +17040,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17050,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17090,7 +17090,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17112,7 +17112,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17134,7 +17134,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17164,7 +17164,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17172,7 +17172,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17182,7 +17182,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17192,7 +17192,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17208,7 +17208,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17297,7 +17297,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17319,7 +17319,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17342,7 +17342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17377,7 +17377,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17412,7 +17412,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17447,7 +17447,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17499,193 +17499,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17855,7 +17855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -17989,7 +17989,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18337,7 +18337,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18511,7 +18511,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18685,7 +18685,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18859,7 +18859,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19033,7 +19033,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19207,7 +19207,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19381,7 +19381,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19555,7 +19555,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19729,7 +19729,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19903,7 +19903,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20077,7 +20077,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20251,7 +20251,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20425,7 +20425,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20599,7 +20599,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20773,7 +20773,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20947,7 +20947,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21121,7 +21121,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21295,7 +21295,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21469,7 +21469,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21643,7 +21643,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21817,7 +21817,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -21991,7 +21991,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22165,7 +22165,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22339,7 +22339,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22513,7 +22513,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22687,7 +22687,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22861,7 +22861,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23035,7 +23035,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23209,7 +23209,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23385,18 +23385,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23409,7 +23409,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23430,7 +23430,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-02-27
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D0EA38-9ECF-4570-9F91-4D0BF44696CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3C0081-1DEF-4FE0-B944-90A3B8A1BED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -2981,34 +2981,34 @@
           <cell r="H60">
             <v>46078</v>
           </cell>
-          <cell r="I60" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J60" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K60" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L60" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I60">
+            <v>3.85E-2</v>
+          </cell>
+          <cell r="J60">
+            <v>4.19E-2</v>
+          </cell>
+          <cell r="K60">
+            <v>4.4600000000000001E-2</v>
+          </cell>
+          <cell r="L60">
+            <v>4.7300000000000002E-2</v>
           </cell>
         </row>
         <row r="61">
           <cell r="H61">
             <v>46079</v>
           </cell>
-          <cell r="I61" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J61" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K61" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L61" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I61">
+            <v>3.8600000000000002E-2</v>
+          </cell>
+          <cell r="J61">
+            <v>4.2000000000000003E-2</v>
+          </cell>
+          <cell r="K61">
+            <v>4.4600000000000001E-2</v>
+          </cell>
+          <cell r="L61">
+            <v>4.7399999999999998E-2</v>
           </cell>
         </row>
         <row r="62">
@@ -9818,21 +9818,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
       </c>
-      <c r="B59" s="17" t="str">
+      <c r="B59" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I60</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C59" s="47" t="str">
+        <v>3.85E-2</v>
+      </c>
+      <c r="C59" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J60</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D59" s="47" t="str">
+        <v>4.19E-2</v>
+      </c>
+      <c r="D59" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K60</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E59" s="5" t="str">
+        <v>4.4600000000000001E-2</v>
+      </c>
+      <c r="E59" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L60</f>
-        <v xml:space="preserve"> </v>
+        <v>4.7300000000000002E-2</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -9840,21 +9840,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
       </c>
-      <c r="B60" s="17" t="str">
+      <c r="B60" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I61</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C60" s="47" t="str">
+        <v>3.8600000000000002E-2</v>
+      </c>
+      <c r="C60" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J61</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D60" s="47" t="str">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="D60" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K61</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E60" s="5" t="str">
+        <v>4.4600000000000001E-2</v>
+      </c>
+      <c r="E60" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L61</f>
-        <v xml:space="preserve"> </v>
+        <v>4.7399999999999998E-2</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-02-28
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3C0081-1DEF-4FE0-B944-90A3B8A1BED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9BFF606-6E92-4FFB-B115-F9D29E9DFF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2720" yWindow="2700" windowWidth="18720" windowHeight="11660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3015,17 +3015,17 @@
           <cell r="H62">
             <v>46080</v>
           </cell>
-          <cell r="I62" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J62" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K62" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L62" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I62">
+            <v>3.8399999999999997E-2</v>
+          </cell>
+          <cell r="J62">
+            <v>4.1799999999999997E-2</v>
+          </cell>
+          <cell r="K62">
+            <v>4.4499999999999998E-2</v>
+          </cell>
+          <cell r="L62">
+            <v>4.7300000000000002E-2</v>
           </cell>
         </row>
         <row r="63">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,9 +8346,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8381,9 +8398,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8559,16 +8593,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8577,7 +8611,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8586,7 +8620,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8603,7 +8637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8625,7 +8659,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8647,7 +8681,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8669,7 +8703,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8691,7 +8725,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8713,7 +8747,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8735,7 +8769,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8757,7 +8791,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8779,7 +8813,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8801,7 +8835,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8823,7 +8857,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8845,7 +8879,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8867,7 +8901,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8889,7 +8923,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8911,7 +8945,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8933,7 +8967,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8955,7 +8989,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8977,7 +9011,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -8999,7 +9033,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9021,7 +9055,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9043,7 +9077,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9065,7 +9099,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9087,7 +9121,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9109,7 +9143,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9131,7 +9165,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9153,7 +9187,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9175,7 +9209,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9197,7 +9231,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9219,7 +9253,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9241,7 +9275,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9263,7 +9297,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9285,7 +9319,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9307,7 +9341,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9329,7 +9363,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9351,7 +9385,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9373,7 +9407,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9395,7 +9429,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9417,7 +9451,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9439,7 +9473,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9461,7 +9495,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9483,7 +9517,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9505,7 +9539,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9527,7 +9561,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9549,7 +9583,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9571,7 +9605,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9593,7 +9627,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9615,7 +9649,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9637,7 +9671,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9659,7 +9693,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9681,7 +9715,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9703,7 +9737,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9725,7 +9759,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9747,7 +9781,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9769,7 +9803,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9791,7 +9825,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9813,7 +9847,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9835,7 +9869,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9857,29 +9891,29 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
       </c>
-      <c r="B61" s="17" t="str">
+      <c r="B61" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I62</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C61" s="47" t="str">
+        <v>3.8399999999999997E-2</v>
+      </c>
+      <c r="C61" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J62</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D61" s="47" t="str">
+        <v>4.1799999999999997E-2</v>
+      </c>
+      <c r="D61" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K62</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E61" s="5" t="str">
+        <v>4.4499999999999998E-2</v>
+      </c>
+      <c r="E61" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L62</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.7300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9901,7 +9935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9923,7 +9957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9945,7 +9979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9967,7 +10001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -9989,7 +10023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10011,7 +10045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10033,7 +10067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10055,7 +10089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10077,7 +10111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10099,7 +10133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10121,7 +10155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10143,7 +10177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10165,7 +10199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10187,7 +10221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10209,7 +10243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10231,7 +10265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10253,7 +10287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10275,7 +10309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10297,7 +10331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10319,7 +10353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10341,7 +10375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10363,7 +10397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10385,7 +10419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10407,7 +10441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10429,7 +10463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10451,7 +10485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10473,7 +10507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10495,7 +10529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10517,7 +10551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10539,7 +10573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10561,7 +10595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10583,7 +10617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10605,7 +10639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10627,7 +10661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10649,7 +10683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10671,7 +10705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10693,7 +10727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10715,7 +10749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10737,7 +10771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10759,7 +10793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10781,7 +10815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10803,7 +10837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10825,7 +10859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10847,7 +10881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10869,7 +10903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10891,7 +10925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10913,7 +10947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10935,7 +10969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10957,7 +10991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10979,7 +11013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11001,7 +11035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11023,7 +11057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11045,7 +11079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11067,7 +11101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11089,7 +11123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11111,7 +11145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11133,7 +11167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11155,7 +11189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11177,7 +11211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11199,7 +11233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11221,7 +11255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11243,7 +11277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11265,7 +11299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11287,7 +11321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11309,7 +11343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11331,7 +11365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11353,7 +11387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11375,7 +11409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11397,7 +11431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11419,7 +11453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11441,7 +11475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11463,7 +11497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11485,7 +11519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11507,7 +11541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11529,7 +11563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11551,7 +11585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11573,7 +11607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11595,7 +11629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11617,7 +11651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11639,7 +11673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11661,7 +11695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11683,7 +11717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11705,7 +11739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11727,7 +11761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11749,7 +11783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11771,7 +11805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11793,7 +11827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11815,7 +11849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11837,7 +11871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11859,7 +11893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11881,7 +11915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11903,7 +11937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11925,7 +11959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11947,7 +11981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11969,7 +12003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -11991,7 +12025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12013,7 +12047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12035,7 +12069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12057,7 +12091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12079,7 +12113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12101,7 +12135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12123,7 +12157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12145,7 +12179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12167,7 +12201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12189,7 +12223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12211,7 +12245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12233,7 +12267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12255,7 +12289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12277,7 +12311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12299,7 +12333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12321,7 +12355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12343,7 +12377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12365,7 +12399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12387,7 +12421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12409,7 +12443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12431,7 +12465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12453,7 +12487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12475,7 +12509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12497,7 +12531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12519,7 +12553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12541,7 +12575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12563,7 +12597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12585,7 +12619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12607,7 +12641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12629,7 +12663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12651,7 +12685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12673,7 +12707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12695,7 +12729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12717,7 +12751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12739,7 +12773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12761,7 +12795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12783,7 +12817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12805,7 +12839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12827,7 +12861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12849,7 +12883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12871,7 +12905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12893,7 +12927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12915,7 +12949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12937,7 +12971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12959,7 +12993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -12981,7 +13015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13003,7 +13037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13025,7 +13059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13047,7 +13081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13069,7 +13103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13091,7 +13125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13113,7 +13147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13135,7 +13169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13157,7 +13191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13179,7 +13213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13201,7 +13235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13223,7 +13257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13245,7 +13279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13267,7 +13301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13289,7 +13323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13311,7 +13345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13333,7 +13367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13355,7 +13389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13377,7 +13411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13399,7 +13433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13421,7 +13455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13443,7 +13477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13465,7 +13499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13487,7 +13521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13509,7 +13543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13531,7 +13565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13553,7 +13587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13575,7 +13609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13597,7 +13631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13619,7 +13653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13641,7 +13675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13663,7 +13697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13685,7 +13719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13707,7 +13741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13729,7 +13763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13751,7 +13785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13773,7 +13807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13795,7 +13829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13817,7 +13851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13839,7 +13873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13861,7 +13895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13883,7 +13917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13905,7 +13939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13927,7 +13961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13949,7 +13983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13971,7 +14005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -13993,7 +14027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14015,7 +14049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14037,7 +14071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14059,7 +14093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14081,7 +14115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14103,7 +14137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14125,7 +14159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14147,7 +14181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14169,7 +14203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14191,7 +14225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14213,7 +14247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14235,7 +14269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14257,7 +14291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14279,7 +14313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14301,7 +14335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14323,7 +14357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14345,7 +14379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14367,7 +14401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14389,7 +14423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14411,7 +14445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14433,7 +14467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14455,7 +14489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14477,7 +14511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14499,7 +14533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14521,7 +14555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14543,7 +14577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14565,7 +14599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14587,7 +14621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14609,7 +14643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14631,7 +14665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14653,7 +14687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14675,7 +14709,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14697,7 +14731,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14719,7 +14753,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14741,7 +14775,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14763,7 +14797,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14785,7 +14819,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14807,7 +14841,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14829,7 +14863,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14851,7 +14885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14873,7 +14907,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14895,7 +14929,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14917,7 +14951,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14939,7 +14973,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14961,7 +14995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -14983,7 +15017,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15005,7 +15039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15027,7 +15061,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15049,7 +15083,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15071,7 +15105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15093,7 +15127,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15115,7 +15149,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15137,7 +15171,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15159,7 +15193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15181,7 +15215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15203,7 +15237,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15225,7 +15259,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15247,7 +15281,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15269,7 +15303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15291,7 +15325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15313,7 +15347,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15335,7 +15369,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15357,7 +15391,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15379,7 +15413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15401,7 +15435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15423,7 +15457,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15445,7 +15479,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15467,7 +15501,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15489,7 +15523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15511,7 +15545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15533,7 +15567,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15555,7 +15589,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15577,7 +15611,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15599,7 +15633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15621,7 +15655,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15643,7 +15677,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15665,7 +15699,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15687,7 +15721,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15709,7 +15743,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15731,7 +15765,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15753,7 +15787,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15775,7 +15809,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15797,7 +15831,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15819,7 +15853,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15841,7 +15875,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15863,7 +15897,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15885,7 +15919,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15907,7 +15941,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15929,7 +15963,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15951,7 +15985,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15973,7 +16007,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -15995,7 +16029,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16017,7 +16051,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16039,7 +16073,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16061,7 +16095,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16083,7 +16117,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16105,7 +16139,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16127,7 +16161,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16149,7 +16183,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16171,7 +16205,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16193,7 +16227,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16215,7 +16249,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16237,7 +16271,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16259,7 +16293,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16281,7 +16315,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16303,7 +16337,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16325,7 +16359,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16347,7 +16381,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16369,7 +16403,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16391,7 +16425,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16413,7 +16447,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16435,7 +16469,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16457,7 +16491,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16479,7 +16513,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16501,7 +16535,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16523,7 +16557,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16545,7 +16579,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16567,7 +16601,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16589,7 +16623,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16611,7 +16645,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16633,7 +16667,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16655,37 +16689,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16701,13 +16735,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16716,14 +16750,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16732,7 +16766,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16741,7 +16775,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16758,7 +16792,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16780,7 +16814,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16802,7 +16836,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16824,7 +16858,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16846,7 +16880,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16863,13 +16897,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16878,7 +16912,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16887,12 +16921,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16901,7 +16935,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16918,7 +16952,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16942,7 +16976,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16966,7 +17000,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -16990,7 +17024,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17014,7 +17048,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17022,7 +17056,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17030,7 +17064,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17040,7 +17074,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17084,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17068,7 +17102,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17090,7 +17124,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17112,7 +17146,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17134,7 +17168,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17156,7 +17190,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17164,7 +17198,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17172,7 +17206,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17182,7 +17216,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17192,7 +17226,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17208,7 +17242,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17228,7 +17262,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17248,7 +17282,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17268,7 +17302,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17288,7 +17322,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17297,7 +17331,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17308,7 +17342,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17319,7 +17353,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17342,7 +17376,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17377,7 +17411,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17412,7 +17446,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17447,7 +17481,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17499,193 +17533,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17855,7 +17889,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -17989,7 +18023,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18163,7 +18197,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18337,7 +18371,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18511,7 +18545,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18685,7 +18719,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18859,7 +18893,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19033,7 +19067,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19207,7 +19241,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19381,7 +19415,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19555,7 +19589,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19729,7 +19763,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19903,7 +19937,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20077,7 +20111,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20251,7 +20285,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20425,7 +20459,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20599,7 +20633,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20773,7 +20807,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20947,7 +20981,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21121,7 +21155,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21295,7 +21329,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21469,7 +21503,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21643,7 +21677,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21817,7 +21851,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -21991,7 +22025,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22165,7 +22199,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22339,7 +22373,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22513,7 +22547,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22687,7 +22721,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22861,7 +22895,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23035,7 +23069,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23209,7 +23243,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23385,18 +23419,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23409,7 +23443,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23430,7 +23464,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-04
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E9459A9-2355-42B0-9F7E-B87035DB57C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFFAF1E5-72FA-404C-84CA-1B3293421F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3083,17 +3083,17 @@
           <cell r="H66">
             <v>46084</v>
           </cell>
-          <cell r="I66" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J66" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K66" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L66" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I66">
+            <v>3.9300000000000002E-2</v>
+          </cell>
+          <cell r="J66">
+            <v>4.2700000000000002E-2</v>
+          </cell>
+          <cell r="K66">
+            <v>4.53E-2</v>
+          </cell>
+          <cell r="L66">
+            <v>4.8099999999999997E-2</v>
           </cell>
         </row>
         <row r="67">
@@ -9950,21 +9950,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
       </c>
-      <c r="B65" s="17" t="str">
+      <c r="B65" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I66</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C65" s="47" t="str">
+        <v>3.9300000000000002E-2</v>
+      </c>
+      <c r="C65" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J66</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D65" s="47" t="str">
+        <v>4.2700000000000002E-2</v>
+      </c>
+      <c r="D65" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K66</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E65" s="5" t="str">
+        <v>4.53E-2</v>
+      </c>
+      <c r="E65" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L66</f>
-        <v xml:space="preserve"> </v>
+        <v>4.8099999999999997E-2</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
@@ -17508,182 +17508,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="61" t="str" cm="1">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="64" t="str">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
@@ -23385,18 +23385,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-05
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFFAF1E5-72FA-404C-84CA-1B3293421F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F11185F-ABC0-45D0-82DD-665B43BA6C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="-110" windowWidth="29020" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30840" yWindow="1710" windowWidth="26175" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3100,17 +3100,17 @@
           <cell r="H67">
             <v>46085</v>
           </cell>
-          <cell r="I67" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J67" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K67" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L67" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I67">
+            <v>3.9399999999999998E-2</v>
+          </cell>
+          <cell r="J67">
+            <v>4.2799999999999998E-2</v>
+          </cell>
+          <cell r="K67">
+            <v>4.5400000000000003E-2</v>
+          </cell>
+          <cell r="L67">
+            <v>4.82E-2</v>
           </cell>
         </row>
         <row r="68">
@@ -8559,16 +8559,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8577,7 +8577,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8586,7 +8586,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8603,7 +8603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8625,7 +8625,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8647,7 +8647,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8669,7 +8669,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8691,7 +8691,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8713,7 +8713,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8735,7 +8735,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8757,7 +8757,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8779,7 +8779,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8801,7 +8801,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8823,7 +8823,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8845,7 +8845,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8867,7 +8867,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8889,7 +8889,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8911,7 +8911,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8933,7 +8933,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8955,7 +8955,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8977,7 +8977,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -8999,7 +8999,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9021,7 +9021,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9043,7 +9043,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9065,7 +9065,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9087,7 +9087,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9109,7 +9109,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9131,7 +9131,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9153,7 +9153,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9175,7 +9175,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9197,7 +9197,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9219,7 +9219,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9241,7 +9241,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9263,7 +9263,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9285,7 +9285,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9307,7 +9307,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9329,7 +9329,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9351,7 +9351,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9373,7 +9373,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9395,7 +9395,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9417,7 +9417,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9439,7 +9439,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9461,7 +9461,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9483,7 +9483,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9505,7 +9505,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9527,7 +9527,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9549,7 +9549,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9571,7 +9571,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9593,7 +9593,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9615,7 +9615,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9637,7 +9637,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9659,7 +9659,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9681,7 +9681,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9703,7 +9703,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9725,7 +9725,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9747,7 +9747,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9769,7 +9769,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9791,7 +9791,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9813,7 +9813,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9835,7 +9835,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9857,7 +9857,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9879,7 +9879,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9901,7 +9901,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9923,7 +9923,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9945,7 +9945,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9967,29 +9967,29 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
       </c>
-      <c r="B66" s="17" t="str">
+      <c r="B66" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I67</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C66" s="47" t="str">
+        <v>3.9399999999999998E-2</v>
+      </c>
+      <c r="C66" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J67</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D66" s="47" t="str">
+        <v>4.2799999999999998E-2</v>
+      </c>
+      <c r="D66" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K67</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E66" s="5" t="str">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="E66" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L67</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4.82E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10011,7 +10011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10033,7 +10033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10055,7 +10055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10077,7 +10077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10099,7 +10099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10121,7 +10121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10143,7 +10143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10165,7 +10165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10187,7 +10187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10209,7 +10209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10231,7 +10231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10253,7 +10253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10275,7 +10275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10297,7 +10297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10319,7 +10319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10341,7 +10341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10363,7 +10363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10385,7 +10385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10407,7 +10407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10429,7 +10429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10451,7 +10451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10473,7 +10473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10495,7 +10495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10517,7 +10517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10539,7 +10539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10561,7 +10561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10583,7 +10583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10605,7 +10605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10627,7 +10627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10649,7 +10649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10671,7 +10671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10693,7 +10693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10715,7 +10715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10737,7 +10737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10759,7 +10759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10781,7 +10781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10803,7 +10803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10825,7 +10825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10847,7 +10847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10869,7 +10869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10891,7 +10891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10913,7 +10913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10935,7 +10935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10957,7 +10957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10979,7 +10979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11001,7 +11001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11023,7 +11023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11045,7 +11045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11067,7 +11067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11089,7 +11089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11111,7 +11111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11133,7 +11133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11155,7 +11155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11177,7 +11177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11199,7 +11199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11221,7 +11221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11243,7 +11243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11265,7 +11265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11287,7 +11287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11309,7 +11309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11331,7 +11331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11353,7 +11353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11375,7 +11375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11397,7 +11397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11419,7 +11419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11441,7 +11441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11463,7 +11463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11485,7 +11485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11507,7 +11507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11529,7 +11529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11551,7 +11551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11573,7 +11573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11595,7 +11595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11617,7 +11617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11639,7 +11639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11661,7 +11661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11683,7 +11683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11705,7 +11705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11727,7 +11727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11749,7 +11749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11771,7 +11771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11793,7 +11793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11815,7 +11815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11837,7 +11837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11859,7 +11859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11881,7 +11881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11903,7 +11903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11925,7 +11925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11947,7 +11947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11969,7 +11969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -11991,7 +11991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12013,7 +12013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12035,7 +12035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12057,7 +12057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12079,7 +12079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12101,7 +12101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12123,7 +12123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12145,7 +12145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12167,7 +12167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12189,7 +12189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12211,7 +12211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12233,7 +12233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12255,7 +12255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12277,7 +12277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12299,7 +12299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12321,7 +12321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12343,7 +12343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12365,7 +12365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12387,7 +12387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12409,7 +12409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12431,7 +12431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12453,7 +12453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12475,7 +12475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12497,7 +12497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12519,7 +12519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12541,7 +12541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12563,7 +12563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12585,7 +12585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12607,7 +12607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12629,7 +12629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12651,7 +12651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12673,7 +12673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12695,7 +12695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12717,7 +12717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12739,7 +12739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12761,7 +12761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12783,7 +12783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12805,7 +12805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12827,7 +12827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12849,7 +12849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12871,7 +12871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12893,7 +12893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12915,7 +12915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12937,7 +12937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12959,7 +12959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -12981,7 +12981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13003,7 +13003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13025,7 +13025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13047,7 +13047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13069,7 +13069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13091,7 +13091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13113,7 +13113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13135,7 +13135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13157,7 +13157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13179,7 +13179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13201,7 +13201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13223,7 +13223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13245,7 +13245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13267,7 +13267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13289,7 +13289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13311,7 +13311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13333,7 +13333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13355,7 +13355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13377,7 +13377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13399,7 +13399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13421,7 +13421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13443,7 +13443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13465,7 +13465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13487,7 +13487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13509,7 +13509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13531,7 +13531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13553,7 +13553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13575,7 +13575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13597,7 +13597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13619,7 +13619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13641,7 +13641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13663,7 +13663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13685,7 +13685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13707,7 +13707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13729,7 +13729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13751,7 +13751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13773,7 +13773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13795,7 +13795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13817,7 +13817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13839,7 +13839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13861,7 +13861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13883,7 +13883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13905,7 +13905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13927,7 +13927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13949,7 +13949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13971,7 +13971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -13993,7 +13993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14015,7 +14015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14037,7 +14037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14059,7 +14059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14081,7 +14081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14103,7 +14103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14125,7 +14125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14147,7 +14147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14169,7 +14169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14191,7 +14191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14213,7 +14213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14235,7 +14235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14257,7 +14257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14279,7 +14279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14301,7 +14301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14323,7 +14323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14345,7 +14345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14367,7 +14367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14389,7 +14389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14411,7 +14411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14433,7 +14433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14455,7 +14455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14477,7 +14477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14499,7 +14499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14521,7 +14521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14543,7 +14543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14565,7 +14565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14587,7 +14587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14609,7 +14609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14631,7 +14631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14653,7 +14653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14675,7 +14675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14697,7 +14697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14719,7 +14719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14741,7 +14741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14763,7 +14763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14785,7 +14785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14807,7 +14807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14829,7 +14829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14851,7 +14851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14873,7 +14873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14895,7 +14895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14917,7 +14917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14939,7 +14939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14961,7 +14961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -14983,7 +14983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15005,7 +15005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15027,7 +15027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15049,7 +15049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15071,7 +15071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15093,7 +15093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15115,7 +15115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15137,7 +15137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15159,7 +15159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15181,7 +15181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15203,7 +15203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15225,7 +15225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15247,7 +15247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15269,7 +15269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15291,7 +15291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15313,7 +15313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15335,7 +15335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15357,7 +15357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15379,7 +15379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15401,7 +15401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15423,7 +15423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15445,7 +15445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15467,7 +15467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15489,7 +15489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15511,7 +15511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15533,7 +15533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15555,7 +15555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15577,7 +15577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15599,7 +15599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15621,7 +15621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15643,7 +15643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15665,7 +15665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15687,7 +15687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15709,7 +15709,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15731,7 +15731,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15753,7 +15753,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15775,7 +15775,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15797,7 +15797,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15819,7 +15819,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15841,7 +15841,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15863,7 +15863,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15885,7 +15885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15907,7 +15907,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15929,7 +15929,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15951,7 +15951,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15973,7 +15973,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -15995,7 +15995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16017,7 +16017,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16039,7 +16039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16061,7 +16061,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16083,7 +16083,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16105,7 +16105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16127,7 +16127,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16149,7 +16149,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16171,7 +16171,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16193,7 +16193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16215,7 +16215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16237,7 +16237,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16259,7 +16259,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16281,7 +16281,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16303,7 +16303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16325,7 +16325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16347,7 +16347,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16369,7 +16369,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16391,7 +16391,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16413,7 +16413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16435,7 +16435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16457,7 +16457,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16479,7 +16479,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16501,7 +16501,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16523,7 +16523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16545,7 +16545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16567,7 +16567,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16589,7 +16589,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16611,7 +16611,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16633,7 +16633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16655,37 +16655,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16701,13 +16701,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16716,14 +16716,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16732,7 +16732,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16741,7 +16741,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16758,7 +16758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16780,7 +16780,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16802,7 +16802,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16824,7 +16824,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16846,7 +16846,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16863,13 +16863,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16878,7 +16878,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16887,12 +16887,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16901,7 +16901,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16918,7 +16918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16942,7 +16942,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16966,7 +16966,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -16990,7 +16990,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17014,7 +17014,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17022,7 +17022,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17030,7 +17030,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17040,7 +17040,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17050,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17090,7 +17090,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17112,7 +17112,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17134,7 +17134,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17164,7 +17164,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17172,7 +17172,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17182,7 +17182,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17192,7 +17192,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17208,7 +17208,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17297,7 +17297,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17319,7 +17319,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17342,7 +17342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17377,7 +17377,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17412,7 +17412,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17447,7 +17447,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17499,193 +17499,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17855,7 +17855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -17989,7 +17989,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18337,7 +18337,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18511,7 +18511,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18685,7 +18685,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18859,7 +18859,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19033,7 +19033,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19207,7 +19207,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19381,7 +19381,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19555,7 +19555,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19729,7 +19729,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19903,7 +19903,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20077,7 +20077,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20251,7 +20251,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20425,7 +20425,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20599,7 +20599,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20773,7 +20773,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20947,7 +20947,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21121,7 +21121,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21295,7 +21295,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21469,7 +21469,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21643,7 +21643,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21817,7 +21817,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -21991,7 +21991,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22165,7 +22165,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22339,7 +22339,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22513,7 +22513,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22687,7 +22687,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22861,7 +22861,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23035,7 +23035,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23209,7 +23209,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23385,18 +23385,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23409,7 +23409,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23430,7 +23430,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-06
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F11185F-ABC0-45D0-82DD-665B43BA6C4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89571D1C-2690-46F5-95C5-071261A345AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30840" yWindow="1710" windowWidth="26175" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3117,17 +3117,17 @@
           <cell r="H68">
             <v>46086</v>
           </cell>
-          <cell r="I68" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J68" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K68" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L68" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I68">
+            <v>3.95E-2</v>
+          </cell>
+          <cell r="J68">
+            <v>4.2799999999999998E-2</v>
+          </cell>
+          <cell r="K68">
+            <v>4.5400000000000003E-2</v>
+          </cell>
+          <cell r="L68">
+            <v>4.8099999999999997E-2</v>
           </cell>
         </row>
         <row r="69">
@@ -8559,16 +8559,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8577,7 +8577,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8586,7 +8586,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8603,7 +8603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8625,7 +8625,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8647,7 +8647,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8669,7 +8669,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8691,7 +8691,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8713,7 +8713,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8735,7 +8735,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8757,7 +8757,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8779,7 +8779,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8801,7 +8801,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8823,7 +8823,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8845,7 +8845,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8867,7 +8867,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8889,7 +8889,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8911,7 +8911,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8933,7 +8933,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8955,7 +8955,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8977,7 +8977,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -8999,7 +8999,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9021,7 +9021,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9043,7 +9043,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9065,7 +9065,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9087,7 +9087,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9109,7 +9109,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9131,7 +9131,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9153,7 +9153,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9175,7 +9175,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9197,7 +9197,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9219,7 +9219,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9241,7 +9241,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9263,7 +9263,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9285,7 +9285,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9307,7 +9307,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9329,7 +9329,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9351,7 +9351,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9373,7 +9373,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9395,7 +9395,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9417,7 +9417,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9439,7 +9439,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9461,7 +9461,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9483,7 +9483,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9505,7 +9505,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9527,7 +9527,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9549,7 +9549,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9571,7 +9571,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9593,7 +9593,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9615,7 +9615,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9637,7 +9637,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9659,7 +9659,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9681,7 +9681,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9703,7 +9703,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9725,7 +9725,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9747,7 +9747,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9769,7 +9769,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9791,7 +9791,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9813,7 +9813,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9835,7 +9835,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9857,7 +9857,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9879,7 +9879,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9901,7 +9901,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9923,7 +9923,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9945,7 +9945,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9967,7 +9967,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -9989,29 +9989,29 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
       </c>
-      <c r="B67" s="17" t="str">
+      <c r="B67" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I68</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C67" s="47" t="str">
+        <v>3.95E-2</v>
+      </c>
+      <c r="C67" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J68</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D67" s="47" t="str">
+        <v>4.2799999999999998E-2</v>
+      </c>
+      <c r="D67" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K68</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E67" s="5" t="str">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="E67" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L68</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.8099999999999997E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10033,7 +10033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10055,7 +10055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10077,7 +10077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10099,7 +10099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10121,7 +10121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10143,7 +10143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10165,7 +10165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10187,7 +10187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10209,7 +10209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10231,7 +10231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10253,7 +10253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10275,7 +10275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10297,7 +10297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10319,7 +10319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10341,7 +10341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10363,7 +10363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10385,7 +10385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10407,7 +10407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10429,7 +10429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10451,7 +10451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10473,7 +10473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10495,7 +10495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10517,7 +10517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10539,7 +10539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10561,7 +10561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10583,7 +10583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10605,7 +10605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10627,7 +10627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10649,7 +10649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10671,7 +10671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10693,7 +10693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10715,7 +10715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10737,7 +10737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10759,7 +10759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10781,7 +10781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10803,7 +10803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10825,7 +10825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10847,7 +10847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10869,7 +10869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10891,7 +10891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10913,7 +10913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10935,7 +10935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10957,7 +10957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10979,7 +10979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11001,7 +11001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11023,7 +11023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11045,7 +11045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11067,7 +11067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11089,7 +11089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11111,7 +11111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11133,7 +11133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11155,7 +11155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11177,7 +11177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11199,7 +11199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11221,7 +11221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11243,7 +11243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11265,7 +11265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11287,7 +11287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11309,7 +11309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11331,7 +11331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11353,7 +11353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11375,7 +11375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11397,7 +11397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11419,7 +11419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11441,7 +11441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11463,7 +11463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11485,7 +11485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11507,7 +11507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11529,7 +11529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11551,7 +11551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11573,7 +11573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11595,7 +11595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11617,7 +11617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11639,7 +11639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11661,7 +11661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11683,7 +11683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11705,7 +11705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11727,7 +11727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11749,7 +11749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11771,7 +11771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11793,7 +11793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11815,7 +11815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11837,7 +11837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11859,7 +11859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11881,7 +11881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11903,7 +11903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11925,7 +11925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11947,7 +11947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11969,7 +11969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -11991,7 +11991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12013,7 +12013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12035,7 +12035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12057,7 +12057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12079,7 +12079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12101,7 +12101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12123,7 +12123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12145,7 +12145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12167,7 +12167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12189,7 +12189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12211,7 +12211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12233,7 +12233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12255,7 +12255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12277,7 +12277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12299,7 +12299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12321,7 +12321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12343,7 +12343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12365,7 +12365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12387,7 +12387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12409,7 +12409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12431,7 +12431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12453,7 +12453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12475,7 +12475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12497,7 +12497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12519,7 +12519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12541,7 +12541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12563,7 +12563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12585,7 +12585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12607,7 +12607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12629,7 +12629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12651,7 +12651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12673,7 +12673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12695,7 +12695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12717,7 +12717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12739,7 +12739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12761,7 +12761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12783,7 +12783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12805,7 +12805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12827,7 +12827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12849,7 +12849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12871,7 +12871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12893,7 +12893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12915,7 +12915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12937,7 +12937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12959,7 +12959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -12981,7 +12981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13003,7 +13003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13025,7 +13025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13047,7 +13047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13069,7 +13069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13091,7 +13091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13113,7 +13113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13135,7 +13135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13157,7 +13157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13179,7 +13179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13201,7 +13201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13223,7 +13223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13245,7 +13245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13267,7 +13267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13289,7 +13289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13311,7 +13311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13333,7 +13333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13355,7 +13355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13377,7 +13377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13399,7 +13399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13421,7 +13421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13443,7 +13443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13465,7 +13465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13487,7 +13487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13509,7 +13509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13531,7 +13531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13553,7 +13553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13575,7 +13575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13597,7 +13597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13619,7 +13619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13641,7 +13641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13663,7 +13663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13685,7 +13685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13707,7 +13707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13729,7 +13729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13751,7 +13751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13773,7 +13773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13795,7 +13795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13817,7 +13817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13839,7 +13839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13861,7 +13861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13883,7 +13883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13905,7 +13905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13927,7 +13927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13949,7 +13949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13971,7 +13971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -13993,7 +13993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14015,7 +14015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14037,7 +14037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14059,7 +14059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14081,7 +14081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14103,7 +14103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14125,7 +14125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14147,7 +14147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14169,7 +14169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14191,7 +14191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14213,7 +14213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14235,7 +14235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14257,7 +14257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14279,7 +14279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14301,7 +14301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14323,7 +14323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14345,7 +14345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14367,7 +14367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14389,7 +14389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14411,7 +14411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14433,7 +14433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14455,7 +14455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14477,7 +14477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14499,7 +14499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14521,7 +14521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14543,7 +14543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14565,7 +14565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14587,7 +14587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14609,7 +14609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14631,7 +14631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14653,7 +14653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14675,7 +14675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14697,7 +14697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14719,7 +14719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14741,7 +14741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14763,7 +14763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14785,7 +14785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14807,7 +14807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14829,7 +14829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14851,7 +14851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14873,7 +14873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14895,7 +14895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14917,7 +14917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14939,7 +14939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14961,7 +14961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -14983,7 +14983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15005,7 +15005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15027,7 +15027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15049,7 +15049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15071,7 +15071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15093,7 +15093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15115,7 +15115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15137,7 +15137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15159,7 +15159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15181,7 +15181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15203,7 +15203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15225,7 +15225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15247,7 +15247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15269,7 +15269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15291,7 +15291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15313,7 +15313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15335,7 +15335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15357,7 +15357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15379,7 +15379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15401,7 +15401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15423,7 +15423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15445,7 +15445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15467,7 +15467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15489,7 +15489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15511,7 +15511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15533,7 +15533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15555,7 +15555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15577,7 +15577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15599,7 +15599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15621,7 +15621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15643,7 +15643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15665,7 +15665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15687,7 +15687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15709,7 +15709,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15731,7 +15731,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15753,7 +15753,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15775,7 +15775,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15797,7 +15797,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15819,7 +15819,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15841,7 +15841,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15863,7 +15863,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15885,7 +15885,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15907,7 +15907,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15929,7 +15929,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15951,7 +15951,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15973,7 +15973,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -15995,7 +15995,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16017,7 +16017,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16039,7 +16039,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16061,7 +16061,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16083,7 +16083,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16105,7 +16105,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16127,7 +16127,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16149,7 +16149,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16171,7 +16171,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16193,7 +16193,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16215,7 +16215,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16237,7 +16237,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16259,7 +16259,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16281,7 +16281,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16303,7 +16303,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16325,7 +16325,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16347,7 +16347,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16369,7 +16369,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16391,7 +16391,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16413,7 +16413,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16435,7 +16435,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16457,7 +16457,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16479,7 +16479,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16501,7 +16501,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16523,7 +16523,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16545,7 +16545,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16567,7 +16567,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16589,7 +16589,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16611,7 +16611,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16633,7 +16633,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16655,37 +16655,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16701,13 +16701,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16716,14 +16716,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16732,7 +16732,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16741,7 +16741,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16758,7 +16758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16780,7 +16780,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16802,7 +16802,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16824,7 +16824,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16846,7 +16846,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16863,13 +16863,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16878,7 +16878,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16887,12 +16887,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16901,7 +16901,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16918,7 +16918,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16942,7 +16942,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16966,7 +16966,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -16990,7 +16990,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17014,7 +17014,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17022,7 +17022,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17030,7 +17030,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17040,7 +17040,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17050,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17090,7 +17090,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17112,7 +17112,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17134,7 +17134,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17156,7 +17156,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17164,7 +17164,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17172,7 +17172,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17182,7 +17182,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17192,7 +17192,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17208,7 +17208,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17297,7 +17297,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17319,7 +17319,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17342,7 +17342,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17377,7 +17377,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17412,7 +17412,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17447,7 +17447,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17499,193 +17499,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17855,7 +17855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -17989,7 +17989,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18337,7 +18337,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18511,7 +18511,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18685,7 +18685,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18859,7 +18859,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19033,7 +19033,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19207,7 +19207,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19381,7 +19381,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19555,7 +19555,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19729,7 +19729,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19903,7 +19903,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20077,7 +20077,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20251,7 +20251,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20425,7 +20425,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20599,7 +20599,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20773,7 +20773,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20947,7 +20947,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21121,7 +21121,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21295,7 +21295,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21469,7 +21469,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21643,7 +21643,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21817,7 +21817,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -21991,7 +21991,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22165,7 +22165,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22339,7 +22339,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22513,7 +22513,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22687,7 +22687,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22861,7 +22861,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23035,7 +23035,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23209,7 +23209,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23385,18 +23385,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23409,7 +23409,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23430,7 +23430,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-07
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89571D1C-2690-46F5-95C5-071261A345AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEE78F6-84FF-4871-A72E-7DCFF61B4463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -703,8 +703,8 @@
       <definedName name="Year_of_Valuation" refersTo="='History Tables'!$D$1"/>
     </definedNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2">
         <row r="1">
           <cell r="D1">
@@ -712,10 +712,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
       <sheetData sheetId="7">
         <row r="6">
           <cell r="Q6">
@@ -954,8 +954,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
       <sheetData sheetId="10">
         <row r="6">
           <cell r="N6">
@@ -1951,11 +1951,6 @@
         </row>
       </sheetData>
       <sheetData sheetId="11">
-        <row r="1">
-          <cell r="D1" t="str">
-            <v>Sec. 3.C.4</v>
-          </cell>
-        </row>
         <row r="14">
           <cell r="D14">
             <v>0.04</v>
@@ -2037,10 +2032,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
       <sheetData sheetId="16">
         <row r="5">
           <cell r="H5">
@@ -3134,17 +3129,17 @@
           <cell r="H69">
             <v>46087</v>
           </cell>
-          <cell r="I69" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J69" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K69" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L69" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I69">
+            <v>0.04</v>
+          </cell>
+          <cell r="J69">
+            <v>4.3299999999999998E-2</v>
+          </cell>
+          <cell r="K69">
+            <v>4.5900000000000003E-2</v>
+          </cell>
+          <cell r="L69">
+            <v>4.8599999999999997E-2</v>
           </cell>
         </row>
         <row r="70">
@@ -8271,9 +8266,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8306,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,9 +8341,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8381,9 +8393,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8555,20 +8584,40 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D4A5F544-68E3-4AE5-9B70-B029EA4CB5DA}">
+  <we:reference id="1c33aa47-7f18-45ef-9463-1a8a868f1e5b" version="1.0.0.2" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200003692" version="1.0.0.2" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8577,7 +8626,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8586,7 +8635,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8603,7 +8652,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8625,7 +8674,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8647,7 +8696,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8669,7 +8718,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8691,7 +8740,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8713,7 +8762,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8735,7 +8784,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8757,7 +8806,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8779,7 +8828,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8801,7 +8850,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8823,7 +8872,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8845,7 +8894,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8867,7 +8916,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8889,7 +8938,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8911,7 +8960,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8933,7 +8982,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8955,7 +9004,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8977,7 +9026,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -8999,7 +9048,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9021,7 +9070,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9043,7 +9092,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9065,7 +9114,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9087,7 +9136,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9109,7 +9158,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9131,7 +9180,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9153,7 +9202,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9175,7 +9224,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9197,7 +9246,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9219,7 +9268,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9241,7 +9290,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9263,7 +9312,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9285,7 +9334,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9307,7 +9356,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9329,7 +9378,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9351,7 +9400,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9373,7 +9422,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9395,7 +9444,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9417,7 +9466,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9439,7 +9488,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9461,7 +9510,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9483,7 +9532,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9505,7 +9554,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9527,7 +9576,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9549,7 +9598,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9571,7 +9620,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9593,7 +9642,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9615,7 +9664,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9637,7 +9686,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9659,7 +9708,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9681,7 +9730,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9703,7 +9752,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9725,7 +9774,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9747,7 +9796,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9769,7 +9818,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9791,7 +9840,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9813,7 +9862,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9835,7 +9884,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9857,7 +9906,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9879,7 +9928,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9901,7 +9950,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9923,7 +9972,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9945,7 +9994,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9967,7 +10016,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -9989,7 +10038,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10011,29 +10060,29 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
       </c>
-      <c r="B68" s="17" t="str">
+      <c r="B68" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I69</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C68" s="47" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="C68" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J69</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D68" s="47" t="str">
+        <v>4.3299999999999998E-2</v>
+      </c>
+      <c r="D68" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K69</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E68" s="5" t="str">
+        <v>4.5900000000000003E-2</v>
+      </c>
+      <c r="E68" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L69</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4.8599999999999997E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10055,7 +10104,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10077,7 +10126,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10099,7 +10148,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10121,7 +10170,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10143,7 +10192,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10165,7 +10214,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10187,7 +10236,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10209,7 +10258,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10231,7 +10280,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10253,7 +10302,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10275,7 +10324,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10297,7 +10346,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10319,7 +10368,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10341,7 +10390,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10363,7 +10412,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10385,7 +10434,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10407,7 +10456,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10429,7 +10478,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10451,7 +10500,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10473,7 +10522,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10495,7 +10544,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10517,7 +10566,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10539,7 +10588,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10561,7 +10610,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10583,7 +10632,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10605,7 +10654,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10627,7 +10676,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10649,7 +10698,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10671,7 +10720,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10693,7 +10742,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10715,7 +10764,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10737,7 +10786,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10759,7 +10808,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10781,7 +10830,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10803,7 +10852,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10825,7 +10874,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10847,7 +10896,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10869,7 +10918,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10891,7 +10940,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10913,7 +10962,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10935,7 +10984,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10957,7 +11006,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10979,7 +11028,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11001,7 +11050,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11023,7 +11072,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11045,7 +11094,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11067,7 +11116,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11089,7 +11138,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11111,7 +11160,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11133,7 +11182,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11155,7 +11204,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11177,7 +11226,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11199,7 +11248,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11221,7 +11270,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11243,7 +11292,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11265,7 +11314,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11287,7 +11336,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11309,7 +11358,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11331,7 +11380,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11353,7 +11402,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11375,7 +11424,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11397,7 +11446,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11419,7 +11468,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11441,7 +11490,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11463,7 +11512,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11485,7 +11534,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11507,7 +11556,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11529,7 +11578,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11551,7 +11600,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11573,7 +11622,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11595,7 +11644,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11617,7 +11666,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11639,7 +11688,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11661,7 +11710,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11683,7 +11732,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11705,7 +11754,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11727,7 +11776,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11749,7 +11798,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11771,7 +11820,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11793,7 +11842,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11815,7 +11864,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11837,7 +11886,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11859,7 +11908,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11881,7 +11930,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11903,7 +11952,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11925,7 +11974,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11947,7 +11996,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11969,7 +12018,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -11991,7 +12040,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12013,7 +12062,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12035,7 +12084,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12057,7 +12106,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12079,7 +12128,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12101,7 +12150,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12123,7 +12172,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12145,7 +12194,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12167,7 +12216,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12189,7 +12238,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12211,7 +12260,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12233,7 +12282,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12255,7 +12304,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12277,7 +12326,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12299,7 +12348,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12321,7 +12370,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12343,7 +12392,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12365,7 +12414,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12387,7 +12436,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12409,7 +12458,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12431,7 +12480,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12453,7 +12502,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12475,7 +12524,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12497,7 +12546,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12519,7 +12568,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12541,7 +12590,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12563,7 +12612,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12585,7 +12634,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12607,7 +12656,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12629,7 +12678,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12651,7 +12700,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12673,7 +12722,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12695,7 +12744,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12717,7 +12766,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12739,7 +12788,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12761,7 +12810,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12783,7 +12832,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12805,7 +12854,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12827,7 +12876,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12849,7 +12898,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12871,7 +12920,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12893,7 +12942,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12915,7 +12964,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12937,7 +12986,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12959,7 +13008,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -12981,7 +13030,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13003,7 +13052,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13025,7 +13074,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13047,7 +13096,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13069,7 +13118,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13091,7 +13140,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13113,7 +13162,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13135,7 +13184,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13157,7 +13206,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13179,7 +13228,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13201,7 +13250,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13223,7 +13272,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13245,7 +13294,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13267,7 +13316,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13289,7 +13338,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13311,7 +13360,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13333,7 +13382,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13355,7 +13404,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13377,7 +13426,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13399,7 +13448,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13421,7 +13470,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13443,7 +13492,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13465,7 +13514,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13487,7 +13536,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13509,7 +13558,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13531,7 +13580,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13553,7 +13602,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13575,7 +13624,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13597,7 +13646,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13619,7 +13668,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13641,7 +13690,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13663,7 +13712,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13685,7 +13734,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13707,7 +13756,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13729,7 +13778,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13751,7 +13800,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13773,7 +13822,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13795,7 +13844,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13817,7 +13866,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13839,7 +13888,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13861,7 +13910,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13883,7 +13932,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13905,7 +13954,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13927,7 +13976,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13949,7 +13998,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13971,7 +14020,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -13993,7 +14042,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14015,7 +14064,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14037,7 +14086,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14059,7 +14108,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14081,7 +14130,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14103,7 +14152,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14125,7 +14174,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14147,7 +14196,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14169,7 +14218,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14191,7 +14240,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14213,7 +14262,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14235,7 +14284,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14257,7 +14306,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14279,7 +14328,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14301,7 +14350,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14323,7 +14372,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14345,7 +14394,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14367,7 +14416,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14389,7 +14438,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14411,7 +14460,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14433,7 +14482,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14455,7 +14504,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14477,7 +14526,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14499,7 +14548,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14521,7 +14570,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14543,7 +14592,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14565,7 +14614,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14587,7 +14636,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14609,7 +14658,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14631,7 +14680,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14653,7 +14702,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14675,7 +14724,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14697,7 +14746,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14719,7 +14768,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14741,7 +14790,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14763,7 +14812,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14785,7 +14834,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14807,7 +14856,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14829,7 +14878,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14851,7 +14900,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14873,7 +14922,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14895,7 +14944,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14917,7 +14966,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14939,7 +14988,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14961,7 +15010,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -14983,7 +15032,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15005,7 +15054,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15027,7 +15076,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15049,7 +15098,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15071,7 +15120,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15093,7 +15142,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15115,7 +15164,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15137,7 +15186,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15159,7 +15208,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15181,7 +15230,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15203,7 +15252,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15225,7 +15274,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15247,7 +15296,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15269,7 +15318,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15291,7 +15340,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15313,7 +15362,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15335,7 +15384,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15357,7 +15406,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15379,7 +15428,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15401,7 +15450,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15423,7 +15472,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15445,7 +15494,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15467,7 +15516,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15489,7 +15538,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15511,7 +15560,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15533,7 +15582,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15555,7 +15604,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15577,7 +15626,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15599,7 +15648,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15621,7 +15670,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15643,7 +15692,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15665,7 +15714,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15687,7 +15736,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15709,7 +15758,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15731,7 +15780,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15753,7 +15802,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15775,7 +15824,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15797,7 +15846,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15819,7 +15868,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15841,7 +15890,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15863,7 +15912,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15885,7 +15934,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15907,7 +15956,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15929,7 +15978,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15951,7 +16000,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15973,7 +16022,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -15995,7 +16044,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16017,7 +16066,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16039,7 +16088,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16061,7 +16110,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16083,7 +16132,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16105,7 +16154,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16127,7 +16176,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16149,7 +16198,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16171,7 +16220,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16193,7 +16242,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16215,7 +16264,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16237,7 +16286,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16259,7 +16308,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16281,7 +16330,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16303,7 +16352,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16325,7 +16374,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16347,7 +16396,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16369,7 +16418,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16391,7 +16440,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16413,7 +16462,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16435,7 +16484,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16457,7 +16506,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16479,7 +16528,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16501,7 +16550,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16523,7 +16572,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16545,7 +16594,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16567,7 +16616,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16589,7 +16638,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16611,7 +16660,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16633,7 +16682,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16655,37 +16704,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16701,13 +16750,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16716,14 +16765,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16732,7 +16781,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16741,7 +16790,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16758,7 +16807,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16780,7 +16829,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16802,7 +16851,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16824,7 +16873,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16846,7 +16895,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16863,13 +16912,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16878,7 +16927,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16887,12 +16936,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16901,7 +16950,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16918,7 +16967,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16942,7 +16991,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16966,7 +17015,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -16990,7 +17039,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17014,7 +17063,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17022,7 +17071,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17030,7 +17079,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17040,7 +17089,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17099,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17068,7 +17117,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17090,7 +17139,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17112,7 +17161,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17134,7 +17183,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17156,7 +17205,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17164,7 +17213,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17172,7 +17221,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17182,7 +17231,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17192,7 +17241,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17208,7 +17257,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17228,7 +17277,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17248,7 +17297,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17268,7 +17317,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17288,7 +17337,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17297,7 +17346,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17308,7 +17357,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17319,7 +17368,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17342,7 +17391,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17377,7 +17426,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17412,7 +17461,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17447,7 +17496,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17499,193 +17548,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17855,7 +17904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -17989,7 +18038,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18163,7 +18212,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18337,7 +18386,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18511,7 +18560,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18685,7 +18734,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18859,7 +18908,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19033,7 +19082,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19207,7 +19256,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19381,7 +19430,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19555,7 +19604,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19729,7 +19778,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19903,7 +19952,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20077,7 +20126,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20251,7 +20300,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20425,7 +20474,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20599,7 +20648,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20773,7 +20822,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20947,7 +20996,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21121,7 +21170,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21295,7 +21344,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21469,7 +21518,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21643,7 +21692,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21817,7 +21866,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -21991,7 +22040,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22165,7 +22214,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22339,7 +22388,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22513,7 +22562,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22687,7 +22736,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22861,7 +22910,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23035,7 +23084,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23209,7 +23258,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23385,18 +23434,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23409,7 +23458,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23430,7 +23479,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-10
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEE78F6-84FF-4871-A72E-7DCFF61B4463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7D892E-729D-40E5-9000-4370A3DB5002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -703,8 +703,8 @@
       <definedName name="Year_of_Valuation" refersTo="='History Tables'!$D$1"/>
     </definedNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
       <sheetData sheetId="2">
         <row r="1">
           <cell r="D1">
@@ -712,10 +712,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
       <sheetData sheetId="7">
         <row r="6">
           <cell r="Q6">
@@ -954,8 +954,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
       <sheetData sheetId="10">
         <row r="6">
           <cell r="N6">
@@ -1951,6 +1951,11 @@
         </row>
       </sheetData>
       <sheetData sheetId="11">
+        <row r="1">
+          <cell r="D1" t="str">
+            <v>Sec. 3.C.4</v>
+          </cell>
+        </row>
         <row r="14">
           <cell r="D14">
             <v>0.04</v>
@@ -2032,10 +2037,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
       <sheetData sheetId="16">
         <row r="5">
           <cell r="H5">
@@ -3146,51 +3151,51 @@
           <cell r="H70">
             <v>46088</v>
           </cell>
-          <cell r="I70" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J70" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K70" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L70" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I70">
+            <v>4.02E-2</v>
+          </cell>
+          <cell r="J70">
+            <v>4.36E-2</v>
+          </cell>
+          <cell r="K70">
+            <v>4.6199999999999998E-2</v>
+          </cell>
+          <cell r="L70">
+            <v>4.8899999999999999E-2</v>
           </cell>
         </row>
         <row r="71">
           <cell r="H71">
             <v>46089</v>
           </cell>
-          <cell r="I71" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J71" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K71" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L71" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I71">
+            <v>4.02E-2</v>
+          </cell>
+          <cell r="J71">
+            <v>4.36E-2</v>
+          </cell>
+          <cell r="K71">
+            <v>4.6199999999999998E-2</v>
+          </cell>
+          <cell r="L71">
+            <v>4.8899999999999999E-2</v>
           </cell>
         </row>
         <row r="72">
           <cell r="H72">
             <v>46090</v>
           </cell>
-          <cell r="I72" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J72" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K72" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L72" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I72">
+            <v>4.02E-2</v>
+          </cell>
+          <cell r="J72">
+            <v>4.36E-2</v>
+          </cell>
+          <cell r="K72">
+            <v>4.6199999999999998E-2</v>
+          </cell>
+          <cell r="L72">
+            <v>4.8899999999999999E-2</v>
           </cell>
         </row>
         <row r="73">
@@ -8266,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8306,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8341,26 +8346,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8393,26 +8381,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8608,16 +8579,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8626,7 +8597,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8635,7 +8606,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8652,7 +8623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8674,7 +8645,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8696,7 +8667,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8718,7 +8689,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8740,7 +8711,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8762,7 +8733,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8784,7 +8755,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8806,7 +8777,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8828,7 +8799,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8850,7 +8821,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8872,7 +8843,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8894,7 +8865,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8916,7 +8887,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8938,7 +8909,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8960,7 +8931,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8982,7 +8953,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -9004,7 +8975,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -9026,7 +8997,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9048,7 +9019,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9070,7 +9041,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9092,7 +9063,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9114,7 +9085,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9136,7 +9107,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9158,7 +9129,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9180,7 +9151,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9202,7 +9173,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9224,7 +9195,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9246,7 +9217,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9268,7 +9239,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9290,7 +9261,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9312,7 +9283,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9334,7 +9305,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9356,7 +9327,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9378,7 +9349,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9400,7 +9371,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9422,7 +9393,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9444,7 +9415,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9466,7 +9437,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9488,7 +9459,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9510,7 +9481,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9532,7 +9503,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9554,7 +9525,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9576,7 +9547,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9598,7 +9569,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9620,7 +9591,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9642,7 +9613,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9664,7 +9635,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9686,7 +9657,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9708,7 +9679,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9730,7 +9701,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9752,7 +9723,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9774,7 +9745,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9796,7 +9767,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9818,7 +9789,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9840,7 +9811,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9862,7 +9833,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9884,7 +9855,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9906,7 +9877,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9928,7 +9899,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9950,7 +9921,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9972,7 +9943,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9994,7 +9965,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -10016,7 +9987,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10038,7 +10009,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10060,7 +10031,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10082,73 +10053,73 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
       </c>
-      <c r="B69" s="17" t="str">
+      <c r="B69" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I70</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C69" s="47" t="str">
+        <v>4.02E-2</v>
+      </c>
+      <c r="C69" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J70</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D69" s="47" t="str">
+        <v>4.36E-2</v>
+      </c>
+      <c r="D69" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K70</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E69" s="5" t="str">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="E69" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L70</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.8899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
       </c>
-      <c r="B70" s="17" t="str">
+      <c r="B70" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I71</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C70" s="47" t="str">
+        <v>4.02E-2</v>
+      </c>
+      <c r="C70" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J71</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D70" s="47" t="str">
+        <v>4.36E-2</v>
+      </c>
+      <c r="D70" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K71</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E70" s="5" t="str">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="E70" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L71</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.8899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
       </c>
-      <c r="B71" s="17" t="str">
+      <c r="B71" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I72</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C71" s="47" t="str">
+        <v>4.02E-2</v>
+      </c>
+      <c r="C71" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J72</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D71" s="47" t="str">
+        <v>4.36E-2</v>
+      </c>
+      <c r="D71" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K72</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E71" s="5" t="str">
+        <v>4.6199999999999998E-2</v>
+      </c>
+      <c r="E71" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L72</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+        <v>4.8899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10170,7 +10141,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10192,7 +10163,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10214,7 +10185,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10236,7 +10207,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10258,7 +10229,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10280,7 +10251,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10302,7 +10273,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10324,7 +10295,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10346,7 +10317,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10368,7 +10339,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10390,7 +10361,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10412,7 +10383,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10434,7 +10405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10456,7 +10427,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10478,7 +10449,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10500,7 +10471,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10522,7 +10493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10544,7 +10515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10566,7 +10537,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10588,7 +10559,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10610,7 +10581,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10632,7 +10603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10654,7 +10625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10676,7 +10647,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10698,7 +10669,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10720,7 +10691,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10742,7 +10713,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10764,7 +10735,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10786,7 +10757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10808,7 +10779,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10830,7 +10801,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10852,7 +10823,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10874,7 +10845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10896,7 +10867,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10918,7 +10889,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10940,7 +10911,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10962,7 +10933,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10984,7 +10955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -11006,7 +10977,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -11028,7 +10999,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11050,7 +11021,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11072,7 +11043,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11094,7 +11065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11116,7 +11087,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11138,7 +11109,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11160,7 +11131,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11182,7 +11153,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11204,7 +11175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11226,7 +11197,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11248,7 +11219,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11270,7 +11241,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11292,7 +11263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11314,7 +11285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11336,7 +11307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11358,7 +11329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11380,7 +11351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11402,7 +11373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11424,7 +11395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11446,7 +11417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11468,7 +11439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11490,7 +11461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11512,7 +11483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11534,7 +11505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11556,7 +11527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11578,7 +11549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11600,7 +11571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11622,7 +11593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11644,7 +11615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11666,7 +11637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11688,7 +11659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11710,7 +11681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11732,7 +11703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11754,7 +11725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11776,7 +11747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11798,7 +11769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11820,7 +11791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11842,7 +11813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11864,7 +11835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11886,7 +11857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11908,7 +11879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11930,7 +11901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11952,7 +11923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11974,7 +11945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11996,7 +11967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -12018,7 +11989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12040,7 +12011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12062,7 +12033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12084,7 +12055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12106,7 +12077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12128,7 +12099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12150,7 +12121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12172,7 +12143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12194,7 +12165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12216,7 +12187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12238,7 +12209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12260,7 +12231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12282,7 +12253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12304,7 +12275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12326,7 +12297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12348,7 +12319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12370,7 +12341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12392,7 +12363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12414,7 +12385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12436,7 +12407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12458,7 +12429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12480,7 +12451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12502,7 +12473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12524,7 +12495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12546,7 +12517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12568,7 +12539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12590,7 +12561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12612,7 +12583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12634,7 +12605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12656,7 +12627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12678,7 +12649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12700,7 +12671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12722,7 +12693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12744,7 +12715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12766,7 +12737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12788,7 +12759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12810,7 +12781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12832,7 +12803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12854,7 +12825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12876,7 +12847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12898,7 +12869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12920,7 +12891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12942,7 +12913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12964,7 +12935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12986,7 +12957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -13008,7 +12979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13030,7 +13001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13052,7 +13023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13074,7 +13045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13096,7 +13067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13118,7 +13089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13140,7 +13111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13162,7 +13133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13184,7 +13155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13206,7 +13177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13228,7 +13199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13250,7 +13221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13272,7 +13243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13294,7 +13265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13316,7 +13287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13338,7 +13309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13360,7 +13331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13382,7 +13353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13404,7 +13375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13426,7 +13397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13448,7 +13419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13470,7 +13441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13492,7 +13463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13514,7 +13485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13536,7 +13507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13558,7 +13529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13580,7 +13551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13602,7 +13573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13624,7 +13595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13646,7 +13617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13668,7 +13639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13690,7 +13661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13712,7 +13683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13734,7 +13705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13756,7 +13727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13778,7 +13749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13800,7 +13771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13822,7 +13793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13844,7 +13815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13866,7 +13837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13888,7 +13859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13910,7 +13881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13932,7 +13903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13954,7 +13925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13976,7 +13947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13998,7 +13969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -14020,7 +13991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14042,7 +14013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14064,7 +14035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14086,7 +14057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14108,7 +14079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14130,7 +14101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14152,7 +14123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14174,7 +14145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14196,7 +14167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14218,7 +14189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14240,7 +14211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14262,7 +14233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14284,7 +14255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14306,7 +14277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14328,7 +14299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14350,7 +14321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14372,7 +14343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14394,7 +14365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14416,7 +14387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14438,7 +14409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14460,7 +14431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14482,7 +14453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14504,7 +14475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14526,7 +14497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14548,7 +14519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14570,7 +14541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14592,7 +14563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14614,7 +14585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14636,7 +14607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14658,7 +14629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14680,7 +14651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14702,7 +14673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14724,7 +14695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14746,7 +14717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14768,7 +14739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14790,7 +14761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14812,7 +14783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14834,7 +14805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14856,7 +14827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14878,7 +14849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14900,7 +14871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14922,7 +14893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14944,7 +14915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14966,7 +14937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14988,7 +14959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -15010,7 +14981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15032,7 +15003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15054,7 +15025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15076,7 +15047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15098,7 +15069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15120,7 +15091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15142,7 +15113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15164,7 +15135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15186,7 +15157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15208,7 +15179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15230,7 +15201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15252,7 +15223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15274,7 +15245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15296,7 +15267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15318,7 +15289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15340,7 +15311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15362,7 +15333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15384,7 +15355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15406,7 +15377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15428,7 +15399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15450,7 +15421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15472,7 +15443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15494,7 +15465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15516,7 +15487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15538,7 +15509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15560,7 +15531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15582,7 +15553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15604,7 +15575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15626,7 +15597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15648,7 +15619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15670,7 +15641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15692,7 +15663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15714,7 +15685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15736,7 +15707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15758,7 +15729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15780,7 +15751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15802,7 +15773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15824,7 +15795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15846,7 +15817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15868,7 +15839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15890,7 +15861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15912,7 +15883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15934,7 +15905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15956,7 +15927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15978,7 +15949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -16000,7 +15971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -16022,7 +15993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16044,7 +16015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16066,7 +16037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16088,7 +16059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16110,7 +16081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16132,7 +16103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16154,7 +16125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16176,7 +16147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16198,7 +16169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16220,7 +16191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16242,7 +16213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16264,7 +16235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16286,7 +16257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16308,7 +16279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16330,7 +16301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16352,7 +16323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16374,7 +16345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16396,7 +16367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16418,7 +16389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16440,7 +16411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16462,7 +16433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16484,7 +16455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16506,7 +16477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16528,7 +16499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16550,7 +16521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16572,7 +16543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16594,7 +16565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16616,7 +16587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16638,7 +16609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16660,7 +16631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16682,7 +16653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16704,37 +16675,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16750,13 +16721,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16765,14 +16736,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16781,7 +16752,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16790,7 +16761,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16807,7 +16778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16829,7 +16800,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16851,7 +16822,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16873,7 +16844,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16895,7 +16866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16912,13 +16883,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16927,7 +16898,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16936,12 +16907,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16950,7 +16921,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16967,7 +16938,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16991,7 +16962,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -17015,7 +16986,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17039,7 +17010,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17063,7 +17034,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17071,7 +17042,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17079,7 +17050,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17089,7 +17060,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17099,7 +17070,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17117,7 +17088,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17139,7 +17110,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17161,7 +17132,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17183,7 +17154,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17205,7 +17176,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17213,7 +17184,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17221,7 +17192,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17231,7 +17202,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17241,7 +17212,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17257,7 +17228,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17277,7 +17248,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17297,7 +17268,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17317,7 +17288,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17337,7 +17308,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17346,7 +17317,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17357,7 +17328,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17368,7 +17339,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17391,7 +17362,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17426,7 +17397,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17461,7 +17432,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17496,7 +17467,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17548,193 +17519,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17904,7 +17875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18038,7 +18009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18212,7 +18183,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18386,7 +18357,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18560,7 +18531,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18734,7 +18705,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18908,7 +18879,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19082,7 +19053,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19256,7 +19227,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19430,7 +19401,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19604,7 +19575,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19778,7 +19749,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19952,7 +19923,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20126,7 +20097,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20300,7 +20271,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20474,7 +20445,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20648,7 +20619,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20822,7 +20793,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20996,7 +20967,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21170,7 +21141,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21344,7 +21315,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21518,7 +21489,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21692,7 +21663,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21866,7 +21837,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22040,7 +22011,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22214,7 +22185,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22388,7 +22359,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22562,7 +22533,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22736,7 +22707,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22910,7 +22881,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23084,7 +23055,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23258,7 +23229,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23434,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23458,7 +23429,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23479,7 +23450,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-11
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7D892E-729D-40E5-9000-4370A3DB5002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6A033C-887C-4B83-AFC6-50CCF08EA3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3202,17 +3202,17 @@
           <cell r="H73">
             <v>46091</v>
           </cell>
-          <cell r="I73" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J73" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K73" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L73" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I73">
+            <v>0.04</v>
+          </cell>
+          <cell r="J73">
+            <v>4.3299999999999998E-2</v>
+          </cell>
+          <cell r="K73">
+            <v>4.58E-2</v>
+          </cell>
+          <cell r="L73">
+            <v>4.8500000000000001E-2</v>
           </cell>
         </row>
         <row r="74">
@@ -8579,16 +8579,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8597,7 +8597,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8606,7 +8606,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8645,7 +8645,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8667,7 +8667,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8689,7 +8689,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8711,7 +8711,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8733,7 +8733,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8755,7 +8755,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8777,7 +8777,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8799,7 +8799,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8821,7 +8821,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8843,7 +8843,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8865,7 +8865,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8887,7 +8887,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8909,7 +8909,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8931,7 +8931,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8953,7 +8953,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8975,7 +8975,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8997,7 +8997,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9019,7 +9019,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9041,7 +9041,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9063,7 +9063,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9085,7 +9085,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9107,7 +9107,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9129,7 +9129,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9151,7 +9151,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9173,7 +9173,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9195,7 +9195,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9217,7 +9217,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9239,7 +9239,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9261,7 +9261,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9283,7 +9283,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9305,7 +9305,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9327,7 +9327,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9349,7 +9349,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9371,7 +9371,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9393,7 +9393,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9415,7 +9415,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9437,7 +9437,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9459,7 +9459,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9481,7 +9481,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9503,7 +9503,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9525,7 +9525,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9547,7 +9547,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9569,7 +9569,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9591,7 +9591,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9613,7 +9613,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9635,7 +9635,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9657,7 +9657,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9679,7 +9679,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9701,7 +9701,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9723,7 +9723,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9745,7 +9745,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9767,7 +9767,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9789,7 +9789,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9811,7 +9811,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9833,7 +9833,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9855,7 +9855,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9877,7 +9877,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9899,7 +9899,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9921,7 +9921,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9943,7 +9943,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9965,7 +9965,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9987,7 +9987,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10009,7 +10009,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10031,7 +10031,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10053,7 +10053,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10075,7 +10075,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10097,7 +10097,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10119,29 +10119,29 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
       </c>
-      <c r="B72" s="17" t="str">
+      <c r="B72" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I73</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C72" s="47" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="C72" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J73</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D72" s="47" t="str">
+        <v>4.3299999999999998E-2</v>
+      </c>
+      <c r="D72" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K73</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E72" s="5" t="str">
+        <v>4.58E-2</v>
+      </c>
+      <c r="E72" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L73</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+        <v>4.8500000000000001E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10163,7 +10163,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10185,7 +10185,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10207,7 +10207,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10229,7 +10229,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10251,7 +10251,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10273,7 +10273,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10295,7 +10295,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10317,7 +10317,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10339,7 +10339,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10361,7 +10361,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10383,7 +10383,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10405,7 +10405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10427,7 +10427,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10449,7 +10449,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10471,7 +10471,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10493,7 +10493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10515,7 +10515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10537,7 +10537,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10559,7 +10559,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10581,7 +10581,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10603,7 +10603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10625,7 +10625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10647,7 +10647,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10669,7 +10669,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10691,7 +10691,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10713,7 +10713,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10735,7 +10735,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10757,7 +10757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10779,7 +10779,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10801,7 +10801,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10823,7 +10823,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10845,7 +10845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10867,7 +10867,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10889,7 +10889,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10911,7 +10911,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10933,7 +10933,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10955,7 +10955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10977,7 +10977,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10999,7 +10999,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11021,7 +11021,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11043,7 +11043,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11065,7 +11065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11087,7 +11087,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11109,7 +11109,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11131,7 +11131,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11153,7 +11153,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11175,7 +11175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11197,7 +11197,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11219,7 +11219,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11241,7 +11241,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11263,7 +11263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11285,7 +11285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11307,7 +11307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11329,7 +11329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11351,7 +11351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11373,7 +11373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11395,7 +11395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11417,7 +11417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11439,7 +11439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11461,7 +11461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11483,7 +11483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11505,7 +11505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11527,7 +11527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11549,7 +11549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11571,7 +11571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11593,7 +11593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11615,7 +11615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11637,7 +11637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11659,7 +11659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11681,7 +11681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11703,7 +11703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11725,7 +11725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11747,7 +11747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11769,7 +11769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11791,7 +11791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11813,7 +11813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11835,7 +11835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11857,7 +11857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11879,7 +11879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11901,7 +11901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11923,7 +11923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11945,7 +11945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11967,7 +11967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11989,7 +11989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12011,7 +12011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12033,7 +12033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12055,7 +12055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12077,7 +12077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12099,7 +12099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12121,7 +12121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12143,7 +12143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12165,7 +12165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12187,7 +12187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12209,7 +12209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12231,7 +12231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12253,7 +12253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12275,7 +12275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12297,7 +12297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12319,7 +12319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12341,7 +12341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12363,7 +12363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12385,7 +12385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12407,7 +12407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12429,7 +12429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12451,7 +12451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12473,7 +12473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12495,7 +12495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12517,7 +12517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12539,7 +12539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12561,7 +12561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12583,7 +12583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12605,7 +12605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12627,7 +12627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12649,7 +12649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12671,7 +12671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12693,7 +12693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12715,7 +12715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12737,7 +12737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12759,7 +12759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12781,7 +12781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12803,7 +12803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12825,7 +12825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12847,7 +12847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12869,7 +12869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12891,7 +12891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12913,7 +12913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12935,7 +12935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12957,7 +12957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12979,7 +12979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13001,7 +13001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13023,7 +13023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13045,7 +13045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13067,7 +13067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13089,7 +13089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13111,7 +13111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13133,7 +13133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13155,7 +13155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13177,7 +13177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13199,7 +13199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13221,7 +13221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13243,7 +13243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13265,7 +13265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13287,7 +13287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13309,7 +13309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13331,7 +13331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13353,7 +13353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13375,7 +13375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13397,7 +13397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13419,7 +13419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13441,7 +13441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13463,7 +13463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13485,7 +13485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13507,7 +13507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13529,7 +13529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13551,7 +13551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13573,7 +13573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13595,7 +13595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13617,7 +13617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13639,7 +13639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13661,7 +13661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13683,7 +13683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13705,7 +13705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13727,7 +13727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13749,7 +13749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13771,7 +13771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13793,7 +13793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13815,7 +13815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13837,7 +13837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13859,7 +13859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13881,7 +13881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13903,7 +13903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13925,7 +13925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13947,7 +13947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13969,7 +13969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13991,7 +13991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14013,7 +14013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14035,7 +14035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14057,7 +14057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14079,7 +14079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14101,7 +14101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14123,7 +14123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14145,7 +14145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14167,7 +14167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14189,7 +14189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14211,7 +14211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14233,7 +14233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14255,7 +14255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14277,7 +14277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14299,7 +14299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14321,7 +14321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14343,7 +14343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14365,7 +14365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14387,7 +14387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14409,7 +14409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14431,7 +14431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14453,7 +14453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14475,7 +14475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14497,7 +14497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14519,7 +14519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14541,7 +14541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14563,7 +14563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14585,7 +14585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14607,7 +14607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14629,7 +14629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14651,7 +14651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14673,7 +14673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14695,7 +14695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14717,7 +14717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14739,7 +14739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14761,7 +14761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14783,7 +14783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14805,7 +14805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14827,7 +14827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14849,7 +14849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14871,7 +14871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14893,7 +14893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14915,7 +14915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14937,7 +14937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14959,7 +14959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14981,7 +14981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15003,7 +15003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15025,7 +15025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15047,7 +15047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15069,7 +15069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15091,7 +15091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15113,7 +15113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15135,7 +15135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15157,7 +15157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15179,7 +15179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15201,7 +15201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15223,7 +15223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15245,7 +15245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15267,7 +15267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15289,7 +15289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15311,7 +15311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15333,7 +15333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15355,7 +15355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15377,7 +15377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15399,7 +15399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15421,7 +15421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15443,7 +15443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15465,7 +15465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15487,7 +15487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15509,7 +15509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15531,7 +15531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15553,7 +15553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15575,7 +15575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15597,7 +15597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15619,7 +15619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15641,7 +15641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15663,7 +15663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15685,7 +15685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15707,7 +15707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15729,7 +15729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15751,7 +15751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15773,7 +15773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15795,7 +15795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15817,7 +15817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15839,7 +15839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15861,7 +15861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15883,7 +15883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15905,7 +15905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15927,7 +15927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15949,7 +15949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15971,7 +15971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15993,7 +15993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16015,7 +16015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16037,7 +16037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16059,7 +16059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16081,7 +16081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16103,7 +16103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16125,7 +16125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16147,7 +16147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16169,7 +16169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16191,7 +16191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16213,7 +16213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16235,7 +16235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16257,7 +16257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16279,7 +16279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16301,7 +16301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16323,7 +16323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16345,7 +16345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16367,7 +16367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16389,7 +16389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16411,7 +16411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16433,7 +16433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16455,7 +16455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16477,7 +16477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16499,7 +16499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16521,7 +16521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16543,7 +16543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16565,7 +16565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16587,7 +16587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16609,7 +16609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16631,7 +16631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16653,7 +16653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16675,37 +16675,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16721,13 +16721,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16736,14 +16736,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16752,7 +16752,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16761,7 +16761,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16778,7 +16778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16800,7 +16800,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16822,7 +16822,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16844,7 +16844,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16866,7 +16866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16883,13 +16883,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16898,7 +16898,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16907,12 +16907,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16921,7 +16921,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16938,7 +16938,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16962,7 +16962,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16986,7 +16986,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17010,7 +17010,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17034,7 +17034,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17042,7 +17042,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17050,7 +17050,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17060,7 +17060,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17070,7 +17070,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17088,7 +17088,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17110,7 +17110,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17132,7 +17132,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17154,7 +17154,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17184,7 +17184,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17192,7 +17192,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17202,7 +17202,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17212,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17317,7 +17317,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17328,7 +17328,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17339,7 +17339,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17362,7 +17362,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17397,7 +17397,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17432,7 +17432,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17467,7 +17467,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17519,193 +17519,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17875,7 +17875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18009,7 +18009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18183,7 +18183,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18357,7 +18357,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18531,7 +18531,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18705,7 +18705,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18879,7 +18879,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19053,7 +19053,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19227,7 +19227,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19401,7 +19401,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19575,7 +19575,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19749,7 +19749,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19923,7 +19923,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20097,7 +20097,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20271,7 +20271,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20445,7 +20445,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20619,7 +20619,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20793,7 +20793,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20967,7 +20967,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21141,7 +21141,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21315,7 +21315,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21489,7 +21489,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21663,7 +21663,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21837,7 +21837,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22011,7 +22011,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22185,7 +22185,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22359,7 +22359,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22533,7 +22533,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22707,7 +22707,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22881,7 +22881,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23055,7 +23055,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23229,7 +23229,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23405,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23429,7 +23429,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23450,7 +23450,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-12
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6A033C-887C-4B83-AFC6-50CCF08EA3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A3D726-9218-481F-8C57-D9DCAC5B0731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32535" yWindow="1470" windowWidth="21765" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3219,17 +3219,17 @@
           <cell r="H74">
             <v>46092</v>
           </cell>
-          <cell r="I74" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J74" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K74" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L74" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I74">
+            <v>4.0300000000000002E-2</v>
+          </cell>
+          <cell r="J74">
+            <v>4.3700000000000003E-2</v>
+          </cell>
+          <cell r="K74">
+            <v>4.6300000000000001E-2</v>
+          </cell>
+          <cell r="L74">
+            <v>4.9099999999999998E-2</v>
           </cell>
         </row>
         <row r="75">
@@ -10146,21 +10146,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
       </c>
-      <c r="B73" s="17" t="str">
+      <c r="B73" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I74</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C73" s="47" t="str">
+        <v>4.0300000000000002E-2</v>
+      </c>
+      <c r="C73" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J74</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D73" s="47" t="str">
+        <v>4.3700000000000003E-2</v>
+      </c>
+      <c r="D73" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K74</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E73" s="5" t="str">
+        <v>4.6300000000000001E-2</v>
+      </c>
+      <c r="E73" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L74</f>
-        <v xml:space="preserve"> </v>
+        <v>4.9099999999999998E-2</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -17528,182 +17528,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
@@ -23405,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-13
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3A3D726-9218-481F-8C57-D9DCAC5B0731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09301DA2-EF99-44DF-BD3E-841AE178AE29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32535" yWindow="1470" windowWidth="21765" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3236,17 +3236,17 @@
           <cell r="H75">
             <v>46093</v>
           </cell>
-          <cell r="I75" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J75" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K75" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L75" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I75">
+            <v>4.1099999999999998E-2</v>
+          </cell>
+          <cell r="J75">
+            <v>4.4600000000000001E-2</v>
+          </cell>
+          <cell r="K75">
+            <v>4.7300000000000002E-2</v>
+          </cell>
+          <cell r="L75">
+            <v>5.0099999999999999E-2</v>
           </cell>
         </row>
         <row r="76">
@@ -8579,16 +8579,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8597,7 +8597,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8606,7 +8606,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8645,7 +8645,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8667,7 +8667,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8689,7 +8689,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8711,7 +8711,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8733,7 +8733,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8755,7 +8755,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8777,7 +8777,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8799,7 +8799,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8821,7 +8821,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8843,7 +8843,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8865,7 +8865,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8887,7 +8887,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8909,7 +8909,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8931,7 +8931,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8953,7 +8953,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8975,7 +8975,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8997,7 +8997,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9019,7 +9019,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9041,7 +9041,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9063,7 +9063,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9085,7 +9085,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9107,7 +9107,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9129,7 +9129,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9151,7 +9151,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9173,7 +9173,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9195,7 +9195,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9217,7 +9217,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9239,7 +9239,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9261,7 +9261,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9283,7 +9283,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9305,7 +9305,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9327,7 +9327,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9349,7 +9349,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9371,7 +9371,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9393,7 +9393,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9415,7 +9415,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9437,7 +9437,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9459,7 +9459,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9481,7 +9481,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9503,7 +9503,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9525,7 +9525,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9547,7 +9547,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9569,7 +9569,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9591,7 +9591,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9613,7 +9613,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9635,7 +9635,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9657,7 +9657,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9679,7 +9679,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9701,7 +9701,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9723,7 +9723,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9745,7 +9745,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9767,7 +9767,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9789,7 +9789,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9811,7 +9811,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9833,7 +9833,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9855,7 +9855,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9877,7 +9877,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9899,7 +9899,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9921,7 +9921,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9943,7 +9943,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9965,7 +9965,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9987,7 +9987,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10009,7 +10009,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10031,7 +10031,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10053,7 +10053,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10075,7 +10075,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10097,7 +10097,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10119,7 +10119,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10141,7 +10141,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10163,29 +10163,29 @@
         <v>4.9099999999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
       </c>
-      <c r="B74" s="17" t="str">
+      <c r="B74" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I75</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C74" s="47" t="str">
+        <v>4.1099999999999998E-2</v>
+      </c>
+      <c r="C74" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J75</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D74" s="47" t="str">
+        <v>4.4600000000000001E-2</v>
+      </c>
+      <c r="D74" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K75</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E74" s="5" t="str">
+        <v>4.7300000000000002E-2</v>
+      </c>
+      <c r="E74" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L75</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.0099999999999999E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10207,7 +10207,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10229,7 +10229,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10251,7 +10251,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10273,7 +10273,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10295,7 +10295,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10317,7 +10317,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10339,7 +10339,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10361,7 +10361,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10383,7 +10383,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10405,7 +10405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10427,7 +10427,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10449,7 +10449,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10471,7 +10471,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10493,7 +10493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10515,7 +10515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10537,7 +10537,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10559,7 +10559,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10581,7 +10581,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10603,7 +10603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10625,7 +10625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10647,7 +10647,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10669,7 +10669,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10691,7 +10691,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10713,7 +10713,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10735,7 +10735,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10757,7 +10757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10779,7 +10779,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10801,7 +10801,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10823,7 +10823,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10845,7 +10845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10867,7 +10867,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10889,7 +10889,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10911,7 +10911,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10933,7 +10933,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10955,7 +10955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10977,7 +10977,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10999,7 +10999,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11021,7 +11021,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11043,7 +11043,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11065,7 +11065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11087,7 +11087,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11109,7 +11109,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11131,7 +11131,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11153,7 +11153,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11175,7 +11175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11197,7 +11197,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11219,7 +11219,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11241,7 +11241,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11263,7 +11263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11285,7 +11285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11307,7 +11307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11329,7 +11329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11351,7 +11351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11373,7 +11373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11395,7 +11395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11417,7 +11417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11439,7 +11439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11461,7 +11461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11483,7 +11483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11505,7 +11505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11527,7 +11527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11549,7 +11549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11571,7 +11571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11593,7 +11593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11615,7 +11615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11637,7 +11637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11659,7 +11659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11681,7 +11681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11703,7 +11703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11725,7 +11725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11747,7 +11747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11769,7 +11769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11791,7 +11791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11813,7 +11813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11835,7 +11835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11857,7 +11857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11879,7 +11879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11901,7 +11901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11923,7 +11923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11945,7 +11945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11967,7 +11967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11989,7 +11989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12011,7 +12011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12033,7 +12033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12055,7 +12055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12077,7 +12077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12099,7 +12099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12121,7 +12121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12143,7 +12143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12165,7 +12165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12187,7 +12187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12209,7 +12209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12231,7 +12231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12253,7 +12253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12275,7 +12275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12297,7 +12297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12319,7 +12319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12341,7 +12341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12363,7 +12363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12385,7 +12385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12407,7 +12407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12429,7 +12429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12451,7 +12451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12473,7 +12473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12495,7 +12495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12517,7 +12517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12539,7 +12539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12561,7 +12561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12583,7 +12583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12605,7 +12605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12627,7 +12627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12649,7 +12649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12671,7 +12671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12693,7 +12693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12715,7 +12715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12737,7 +12737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12759,7 +12759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12781,7 +12781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12803,7 +12803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12825,7 +12825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12847,7 +12847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12869,7 +12869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12891,7 +12891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12913,7 +12913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12935,7 +12935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12957,7 +12957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12979,7 +12979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13001,7 +13001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13023,7 +13023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13045,7 +13045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13067,7 +13067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13089,7 +13089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13111,7 +13111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13133,7 +13133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13155,7 +13155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13177,7 +13177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13199,7 +13199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13221,7 +13221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13243,7 +13243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13265,7 +13265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13287,7 +13287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13309,7 +13309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13331,7 +13331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13353,7 +13353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13375,7 +13375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13397,7 +13397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13419,7 +13419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13441,7 +13441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13463,7 +13463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13485,7 +13485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13507,7 +13507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13529,7 +13529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13551,7 +13551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13573,7 +13573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13595,7 +13595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13617,7 +13617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13639,7 +13639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13661,7 +13661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13683,7 +13683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13705,7 +13705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13727,7 +13727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13749,7 +13749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13771,7 +13771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13793,7 +13793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13815,7 +13815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13837,7 +13837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13859,7 +13859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13881,7 +13881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13903,7 +13903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13925,7 +13925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13947,7 +13947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13969,7 +13969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13991,7 +13991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14013,7 +14013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14035,7 +14035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14057,7 +14057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14079,7 +14079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14101,7 +14101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14123,7 +14123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14145,7 +14145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14167,7 +14167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14189,7 +14189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14211,7 +14211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14233,7 +14233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14255,7 +14255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14277,7 +14277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14299,7 +14299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14321,7 +14321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14343,7 +14343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14365,7 +14365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14387,7 +14387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14409,7 +14409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14431,7 +14431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14453,7 +14453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14475,7 +14475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14497,7 +14497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14519,7 +14519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14541,7 +14541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14563,7 +14563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14585,7 +14585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14607,7 +14607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14629,7 +14629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14651,7 +14651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14673,7 +14673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14695,7 +14695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14717,7 +14717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14739,7 +14739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14761,7 +14761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14783,7 +14783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14805,7 +14805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14827,7 +14827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14849,7 +14849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14871,7 +14871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14893,7 +14893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14915,7 +14915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14937,7 +14937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14959,7 +14959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14981,7 +14981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15003,7 +15003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15025,7 +15025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15047,7 +15047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15069,7 +15069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15091,7 +15091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15113,7 +15113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15135,7 +15135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15157,7 +15157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15179,7 +15179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15201,7 +15201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15223,7 +15223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15245,7 +15245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15267,7 +15267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15289,7 +15289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15311,7 +15311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15333,7 +15333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15355,7 +15355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15377,7 +15377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15399,7 +15399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15421,7 +15421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15443,7 +15443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15465,7 +15465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15487,7 +15487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15509,7 +15509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15531,7 +15531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15553,7 +15553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15575,7 +15575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15597,7 +15597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15619,7 +15619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15641,7 +15641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15663,7 +15663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15685,7 +15685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15707,7 +15707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15729,7 +15729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15751,7 +15751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15773,7 +15773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15795,7 +15795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15817,7 +15817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15839,7 +15839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15861,7 +15861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15883,7 +15883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15905,7 +15905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15927,7 +15927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15949,7 +15949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15971,7 +15971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15993,7 +15993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16015,7 +16015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16037,7 +16037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16059,7 +16059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16081,7 +16081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16103,7 +16103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16125,7 +16125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16147,7 +16147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16169,7 +16169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16191,7 +16191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16213,7 +16213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16235,7 +16235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16257,7 +16257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16279,7 +16279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16301,7 +16301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16323,7 +16323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16345,7 +16345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16367,7 +16367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16389,7 +16389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16411,7 +16411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16433,7 +16433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16455,7 +16455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16477,7 +16477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16499,7 +16499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16521,7 +16521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16543,7 +16543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16565,7 +16565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16587,7 +16587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16609,7 +16609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16631,7 +16631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16653,7 +16653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16675,37 +16675,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16721,13 +16721,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16736,14 +16736,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16752,7 +16752,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16761,7 +16761,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16778,7 +16778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16800,7 +16800,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16822,7 +16822,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16844,7 +16844,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16866,7 +16866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16883,13 +16883,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16898,7 +16898,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16907,12 +16907,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16921,7 +16921,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16938,7 +16938,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16962,7 +16962,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16986,7 +16986,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17010,7 +17010,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17034,7 +17034,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17042,7 +17042,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17050,7 +17050,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17060,7 +17060,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17070,7 +17070,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17088,7 +17088,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17110,7 +17110,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17132,7 +17132,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17154,7 +17154,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17184,7 +17184,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17192,7 +17192,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17202,7 +17202,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17212,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17317,7 +17317,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17328,7 +17328,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17339,7 +17339,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17362,7 +17362,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17397,7 +17397,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17432,7 +17432,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17467,7 +17467,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17519,193 +17519,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17875,7 +17875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18009,7 +18009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18183,7 +18183,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18357,7 +18357,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18531,7 +18531,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18705,7 +18705,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18879,7 +18879,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19053,7 +19053,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19227,7 +19227,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19401,7 +19401,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19575,7 +19575,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19749,7 +19749,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19923,7 +19923,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20097,7 +20097,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20271,7 +20271,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20445,7 +20445,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20619,7 +20619,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20793,7 +20793,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20967,7 +20967,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21141,7 +21141,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21315,7 +21315,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21489,7 +21489,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21663,7 +21663,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21837,7 +21837,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22011,7 +22011,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22185,7 +22185,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22359,7 +22359,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22533,7 +22533,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22707,7 +22707,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22881,7 +22881,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23055,7 +23055,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23229,7 +23229,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23405,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23429,7 +23429,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23450,7 +23450,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-14
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09301DA2-EF99-44DF-BD3E-841AE178AE29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59B7DAB-D327-48A9-93EF-145D4ECC115E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3253,17 +3253,17 @@
           <cell r="H76">
             <v>46094</v>
           </cell>
-          <cell r="I76" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J76" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K76" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L76" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I76">
+            <v>4.2200000000000001E-2</v>
+          </cell>
+          <cell r="J76">
+            <v>4.5400000000000003E-2</v>
+          </cell>
+          <cell r="K76">
+            <v>4.8000000000000001E-2</v>
+          </cell>
+          <cell r="L76">
+            <v>5.0700000000000002E-2</v>
           </cell>
         </row>
         <row r="77">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,9 +8346,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8381,9 +8398,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8579,16 +8613,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8597,7 +8631,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8606,7 +8640,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8645,7 +8679,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8667,7 +8701,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8689,7 +8723,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8711,7 +8745,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8733,7 +8767,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8755,7 +8789,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8777,7 +8811,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8799,7 +8833,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8821,7 +8855,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8843,7 +8877,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8865,7 +8899,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8887,7 +8921,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8909,7 +8943,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8931,7 +8965,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8953,7 +8987,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8975,7 +9009,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8997,7 +9031,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9019,7 +9053,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9041,7 +9075,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9063,7 +9097,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9085,7 +9119,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9107,7 +9141,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9129,7 +9163,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9151,7 +9185,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9173,7 +9207,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9195,7 +9229,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9217,7 +9251,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9239,7 +9273,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9261,7 +9295,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9283,7 +9317,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9305,7 +9339,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9327,7 +9361,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9349,7 +9383,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9371,7 +9405,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9393,7 +9427,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9415,7 +9449,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9437,7 +9471,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9459,7 +9493,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9481,7 +9515,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9503,7 +9537,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9525,7 +9559,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9547,7 +9581,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9569,7 +9603,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9591,7 +9625,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9613,7 +9647,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9635,7 +9669,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9657,7 +9691,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9679,7 +9713,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9701,7 +9735,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9723,7 +9757,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9745,7 +9779,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9767,7 +9801,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9789,7 +9823,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9811,7 +9845,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9833,7 +9867,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9855,7 +9889,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9877,7 +9911,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9899,7 +9933,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9921,7 +9955,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9943,7 +9977,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9965,7 +9999,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9987,7 +10021,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10009,7 +10043,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10031,7 +10065,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10053,7 +10087,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10075,7 +10109,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10097,7 +10131,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10119,7 +10153,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10141,7 +10175,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10163,7 +10197,7 @@
         <v>4.9099999999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10185,29 +10219,29 @@
         <v>5.0099999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
       </c>
-      <c r="B75" s="17" t="str">
+      <c r="B75" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I76</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C75" s="47" t="str">
+        <v>4.2200000000000001E-2</v>
+      </c>
+      <c r="C75" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J76</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D75" s="47" t="str">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="D75" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K76</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E75" s="5" t="str">
+        <v>4.8000000000000001E-2</v>
+      </c>
+      <c r="E75" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L76</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+        <v>5.0700000000000002E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10229,7 +10263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10251,7 +10285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10273,7 +10307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10295,7 +10329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10317,7 +10351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10339,7 +10373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10361,7 +10395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10383,7 +10417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10405,7 +10439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10427,7 +10461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10449,7 +10483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10471,7 +10505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10493,7 +10527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10515,7 +10549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10537,7 +10571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10559,7 +10593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10581,7 +10615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10603,7 +10637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10625,7 +10659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10647,7 +10681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10669,7 +10703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10691,7 +10725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10713,7 +10747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10735,7 +10769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10757,7 +10791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10779,7 +10813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10801,7 +10835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10823,7 +10857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10845,7 +10879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10867,7 +10901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10889,7 +10923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10911,7 +10945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10933,7 +10967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10955,7 +10989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10977,7 +11011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10999,7 +11033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11021,7 +11055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11043,7 +11077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11065,7 +11099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11087,7 +11121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11109,7 +11143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11131,7 +11165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11153,7 +11187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11175,7 +11209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11197,7 +11231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11219,7 +11253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11241,7 +11275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11263,7 +11297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11285,7 +11319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11307,7 +11341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11329,7 +11363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11351,7 +11385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11373,7 +11407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11395,7 +11429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11417,7 +11451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11439,7 +11473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11461,7 +11495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11483,7 +11517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11505,7 +11539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11527,7 +11561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11549,7 +11583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11571,7 +11605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11593,7 +11627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11615,7 +11649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11637,7 +11671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11659,7 +11693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11681,7 +11715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11703,7 +11737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11725,7 +11759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11747,7 +11781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11769,7 +11803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11791,7 +11825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11813,7 +11847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11835,7 +11869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11857,7 +11891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11879,7 +11913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11901,7 +11935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11923,7 +11957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11945,7 +11979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11967,7 +12001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11989,7 +12023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12011,7 +12045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12033,7 +12067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12055,7 +12089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12077,7 +12111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12099,7 +12133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12121,7 +12155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12143,7 +12177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12165,7 +12199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12187,7 +12221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12209,7 +12243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12231,7 +12265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12253,7 +12287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12275,7 +12309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12297,7 +12331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12319,7 +12353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12341,7 +12375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12363,7 +12397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12385,7 +12419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12407,7 +12441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12429,7 +12463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12451,7 +12485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12473,7 +12507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12495,7 +12529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12517,7 +12551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12539,7 +12573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12561,7 +12595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12583,7 +12617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12605,7 +12639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12627,7 +12661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12649,7 +12683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12671,7 +12705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12693,7 +12727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12715,7 +12749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12737,7 +12771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12759,7 +12793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12781,7 +12815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12803,7 +12837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12825,7 +12859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12847,7 +12881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12869,7 +12903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12891,7 +12925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12913,7 +12947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12935,7 +12969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12957,7 +12991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12979,7 +13013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13001,7 +13035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13023,7 +13057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13045,7 +13079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13067,7 +13101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13089,7 +13123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13111,7 +13145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13133,7 +13167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13155,7 +13189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13177,7 +13211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13199,7 +13233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13221,7 +13255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13243,7 +13277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13265,7 +13299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13287,7 +13321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13309,7 +13343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13331,7 +13365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13353,7 +13387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13375,7 +13409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13397,7 +13431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13419,7 +13453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13441,7 +13475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13463,7 +13497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13485,7 +13519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13507,7 +13541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13529,7 +13563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13551,7 +13585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13573,7 +13607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13595,7 +13629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13617,7 +13651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13639,7 +13673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13661,7 +13695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13683,7 +13717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13705,7 +13739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13727,7 +13761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13749,7 +13783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13771,7 +13805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13793,7 +13827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13815,7 +13849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13837,7 +13871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13859,7 +13893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13881,7 +13915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13903,7 +13937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13925,7 +13959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13947,7 +13981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13969,7 +14003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13991,7 +14025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14013,7 +14047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14035,7 +14069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14057,7 +14091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14079,7 +14113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14101,7 +14135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14123,7 +14157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14145,7 +14179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14167,7 +14201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14189,7 +14223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14211,7 +14245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14233,7 +14267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14255,7 +14289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14277,7 +14311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14299,7 +14333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14321,7 +14355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14343,7 +14377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14365,7 +14399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14387,7 +14421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14409,7 +14443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14431,7 +14465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14453,7 +14487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14475,7 +14509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14497,7 +14531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14519,7 +14553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14541,7 +14575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14563,7 +14597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14585,7 +14619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14607,7 +14641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14629,7 +14663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14651,7 +14685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14673,7 +14707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14695,7 +14729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14717,7 +14751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14739,7 +14773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14761,7 +14795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14783,7 +14817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14805,7 +14839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14827,7 +14861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14849,7 +14883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14871,7 +14905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14893,7 +14927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14915,7 +14949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14937,7 +14971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14959,7 +14993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14981,7 +15015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15003,7 +15037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15025,7 +15059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15047,7 +15081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15069,7 +15103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15091,7 +15125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15113,7 +15147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15135,7 +15169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15157,7 +15191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15179,7 +15213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15201,7 +15235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15223,7 +15257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15245,7 +15279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15267,7 +15301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15289,7 +15323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15311,7 +15345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15333,7 +15367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15355,7 +15389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15377,7 +15411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15399,7 +15433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15421,7 +15455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15443,7 +15477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15465,7 +15499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15487,7 +15521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15509,7 +15543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15531,7 +15565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15553,7 +15587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15575,7 +15609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15597,7 +15631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15619,7 +15653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15641,7 +15675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15663,7 +15697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15685,7 +15719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15707,7 +15741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15729,7 +15763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15751,7 +15785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15773,7 +15807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15795,7 +15829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15817,7 +15851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15839,7 +15873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15861,7 +15895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15883,7 +15917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15905,7 +15939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15927,7 +15961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15949,7 +15983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15971,7 +16005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15993,7 +16027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16015,7 +16049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16037,7 +16071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16059,7 +16093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16081,7 +16115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16103,7 +16137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16125,7 +16159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16147,7 +16181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16169,7 +16203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16191,7 +16225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16213,7 +16247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16235,7 +16269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16257,7 +16291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16279,7 +16313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16301,7 +16335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16323,7 +16357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16345,7 +16379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16367,7 +16401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16389,7 +16423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16411,7 +16445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16433,7 +16467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16455,7 +16489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16477,7 +16511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16499,7 +16533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16521,7 +16555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16543,7 +16577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16565,7 +16599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16587,7 +16621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16609,7 +16643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16631,7 +16665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16653,7 +16687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16675,37 +16709,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16721,13 +16755,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16736,14 +16770,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16752,7 +16786,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16761,7 +16795,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16778,7 +16812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16800,7 +16834,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16822,7 +16856,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16844,7 +16878,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16866,7 +16900,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16883,13 +16917,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16898,7 +16932,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16907,12 +16941,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16921,7 +16955,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16938,7 +16972,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16962,7 +16996,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16986,7 +17020,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17010,7 +17044,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17034,7 +17068,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17042,7 +17076,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17050,7 +17084,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17060,7 +17094,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17070,7 +17104,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17088,7 +17122,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17110,7 +17144,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17132,7 +17166,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17154,7 +17188,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17176,7 +17210,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17184,7 +17218,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17192,7 +17226,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17202,7 +17236,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17246,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17228,7 +17262,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17248,7 +17282,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17268,7 +17302,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17288,7 +17322,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17308,7 +17342,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17317,7 +17351,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17328,7 +17362,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17339,7 +17373,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17362,7 +17396,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17397,7 +17431,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17432,7 +17466,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17467,7 +17501,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17519,193 +17553,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17875,7 +17909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18009,7 +18043,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18183,7 +18217,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18357,7 +18391,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18531,7 +18565,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18705,7 +18739,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18879,7 +18913,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19053,7 +19087,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19227,7 +19261,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19401,7 +19435,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19575,7 +19609,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19749,7 +19783,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19923,7 +19957,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20097,7 +20131,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20271,7 +20305,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20445,7 +20479,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20619,7 +20653,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20793,7 +20827,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20967,7 +21001,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21141,7 +21175,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21315,7 +21349,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21489,7 +21523,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21663,7 +21697,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21837,7 +21871,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22011,7 +22045,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22185,7 +22219,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22359,7 +22393,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22533,7 +22567,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22707,7 +22741,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22881,7 +22915,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23055,7 +23089,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23229,7 +23263,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23405,18 +23439,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23429,7 +23463,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23450,7 +23484,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-17
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D59B7DAB-D327-48A9-93EF-145D4ECC115E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE1DF8E-056D-4D6B-BED5-B373542E0536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31215" yWindow="2040" windowWidth="21765" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3270,51 +3270,51 @@
           <cell r="H77">
             <v>46095</v>
           </cell>
-          <cell r="I77" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J77" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K77" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L77" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I77">
+            <v>4.2500000000000003E-2</v>
+          </cell>
+          <cell r="J77">
+            <v>4.58E-2</v>
+          </cell>
+          <cell r="K77">
+            <v>4.8399999999999999E-2</v>
+          </cell>
+          <cell r="L77">
+            <v>5.11E-2</v>
           </cell>
         </row>
         <row r="78">
           <cell r="H78">
             <v>46096</v>
           </cell>
-          <cell r="I78" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J78" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K78" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L78" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I78">
+            <v>4.2500000000000003E-2</v>
+          </cell>
+          <cell r="J78">
+            <v>4.58E-2</v>
+          </cell>
+          <cell r="K78">
+            <v>4.8399999999999999E-2</v>
+          </cell>
+          <cell r="L78">
+            <v>5.11E-2</v>
           </cell>
         </row>
         <row r="79">
           <cell r="H79">
             <v>46097</v>
           </cell>
-          <cell r="I79" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J79" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K79" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L79" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I79">
+            <v>4.2500000000000003E-2</v>
+          </cell>
+          <cell r="J79">
+            <v>4.58E-2</v>
+          </cell>
+          <cell r="K79">
+            <v>4.8399999999999999E-2</v>
+          </cell>
+          <cell r="L79">
+            <v>5.11E-2</v>
           </cell>
         </row>
         <row r="80">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,26 +8346,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8398,26 +8381,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -10246,21 +10212,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
       </c>
-      <c r="B76" s="17" t="str">
+      <c r="B76" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I77</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C76" s="47" t="str">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="C76" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J77</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D76" s="47" t="str">
+        <v>4.58E-2</v>
+      </c>
+      <c r="D76" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K77</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E76" s="5" t="str">
+        <v>4.8399999999999999E-2</v>
+      </c>
+      <c r="E76" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L77</f>
-        <v xml:space="preserve"> </v>
+        <v>5.11E-2</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -10268,21 +10234,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
       </c>
-      <c r="B77" s="17" t="str">
+      <c r="B77" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I78</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C77" s="47" t="str">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="C77" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J78</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D77" s="47" t="str">
+        <v>4.58E-2</v>
+      </c>
+      <c r="D77" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K78</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E77" s="5" t="str">
+        <v>4.8399999999999999E-2</v>
+      </c>
+      <c r="E77" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L78</f>
-        <v xml:space="preserve"> </v>
+        <v>5.11E-2</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -10290,21 +10256,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
       </c>
-      <c r="B78" s="17" t="str">
+      <c r="B78" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I79</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C78" s="47" t="str">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="C78" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J79</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D78" s="47" t="str">
+        <v>4.58E-2</v>
+      </c>
+      <c r="D78" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K79</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E78" s="5" t="str">
+        <v>4.8399999999999999E-2</v>
+      </c>
+      <c r="E78" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L79</f>
-        <v xml:space="preserve"> </v>
+        <v>5.11E-2</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -17562,182 +17528,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="str" cm="1">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="str">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
@@ -23439,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-18
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE1DF8E-056D-4D6B-BED5-B373542E0536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6297D282-D6F9-4832-AE40-6D07B143B9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31215" yWindow="2040" windowWidth="21765" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24750" yWindow="1350" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -679,6 +679,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Notes"/>
@@ -3321,17 +3322,17 @@
           <cell r="H80">
             <v>46098</v>
           </cell>
-          <cell r="I80" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J80" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K80" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L80" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I80">
+            <v>4.2000000000000003E-2</v>
+          </cell>
+          <cell r="J80">
+            <v>4.5199999999999997E-2</v>
+          </cell>
+          <cell r="K80">
+            <v>4.7800000000000002E-2</v>
+          </cell>
+          <cell r="L80">
+            <v>5.0500000000000003E-2</v>
           </cell>
         </row>
         <row r="81">
@@ -10278,21 +10279,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
       </c>
-      <c r="B79" s="17" t="str">
+      <c r="B79" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I80</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C79" s="47" t="str">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="C79" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J80</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D79" s="47" t="str">
+        <v>4.5199999999999997E-2</v>
+      </c>
+      <c r="D79" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K80</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E79" s="5" t="str">
+        <v>4.7800000000000002E-2</v>
+      </c>
+      <c r="E79" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L80</f>
-        <v xml:space="preserve"> </v>
+        <v>5.0500000000000003E-2</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -17528,182 +17529,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
@@ -23405,18 +23406,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-19
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6297D282-D6F9-4832-AE40-6D07B143B9FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9AE82C-81A6-4C2D-905A-D9893039DA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24750" yWindow="1350" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29910" yWindow="1440" windowWidth="27420" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -679,7 +679,6 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Notes"/>
@@ -3339,17 +3338,17 @@
           <cell r="H81">
             <v>46099</v>
           </cell>
-          <cell r="I81" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J81" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K81" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L81" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I81">
+            <v>4.1599999999999998E-2</v>
+          </cell>
+          <cell r="J81">
+            <v>4.48E-2</v>
+          </cell>
+          <cell r="K81">
+            <v>4.7399999999999998E-2</v>
+          </cell>
+          <cell r="L81">
+            <v>0.05</v>
           </cell>
         </row>
         <row r="82">
@@ -10301,21 +10300,21 @@
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
       </c>
-      <c r="B80" s="17" t="str">
+      <c r="B80" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I81</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C80" s="47" t="str">
+        <v>4.1599999999999998E-2</v>
+      </c>
+      <c r="C80" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J81</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D80" s="47" t="str">
+        <v>4.48E-2</v>
+      </c>
+      <c r="D80" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K81</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E80" s="5" t="str">
+        <v>4.7399999999999998E-2</v>
+      </c>
+      <c r="E80" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L81</f>
-        <v xml:space="preserve"> </v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -17529,182 +17528,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="str" cm="1">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="str">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
@@ -23406,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-20
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9AE82C-81A6-4C2D-905A-D9893039DA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA7BFF2-3523-4C0C-8630-E9018763D16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29910" yWindow="1440" windowWidth="27420" windowHeight="12810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17565" yWindow="1110" windowWidth="12480" windowHeight="7770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3355,17 +3355,17 @@
           <cell r="H82">
             <v>46100</v>
           </cell>
-          <cell r="I82" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J82" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K82" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L82" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I82">
+            <v>4.2299999999999997E-2</v>
+          </cell>
+          <cell r="J82">
+            <v>4.5400000000000003E-2</v>
+          </cell>
+          <cell r="K82">
+            <v>4.7800000000000002E-2</v>
+          </cell>
+          <cell r="L82">
+            <v>5.04E-2</v>
           </cell>
         </row>
         <row r="83">
@@ -8579,16 +8579,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8597,7 +8597,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8606,7 +8606,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8645,7 +8645,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8667,7 +8667,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8689,7 +8689,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8711,7 +8711,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8733,7 +8733,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8755,7 +8755,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8777,7 +8777,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8799,7 +8799,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8821,7 +8821,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8843,7 +8843,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8865,7 +8865,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8887,7 +8887,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8909,7 +8909,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8931,7 +8931,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8953,7 +8953,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8975,7 +8975,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8997,7 +8997,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9019,7 +9019,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9041,7 +9041,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9063,7 +9063,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9085,7 +9085,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9107,7 +9107,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9129,7 +9129,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9151,7 +9151,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9173,7 +9173,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9195,7 +9195,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9217,7 +9217,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9239,7 +9239,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9261,7 +9261,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9283,7 +9283,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9305,7 +9305,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9327,7 +9327,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9349,7 +9349,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9371,7 +9371,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9393,7 +9393,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9415,7 +9415,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9437,7 +9437,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9459,7 +9459,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9481,7 +9481,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9503,7 +9503,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9525,7 +9525,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9547,7 +9547,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9569,7 +9569,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9591,7 +9591,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9613,7 +9613,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9635,7 +9635,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9657,7 +9657,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9679,7 +9679,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9701,7 +9701,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9723,7 +9723,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9745,7 +9745,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9767,7 +9767,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9789,7 +9789,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9811,7 +9811,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9833,7 +9833,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9855,7 +9855,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9877,7 +9877,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9899,7 +9899,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9921,7 +9921,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9943,7 +9943,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9965,7 +9965,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9987,7 +9987,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10009,7 +10009,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10031,7 +10031,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10053,7 +10053,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10075,7 +10075,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10097,7 +10097,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10119,7 +10119,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10141,7 +10141,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10163,7 +10163,7 @@
         <v>4.9099999999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10185,7 +10185,7 @@
         <v>5.0099999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10207,7 +10207,7 @@
         <v>5.0700000000000002E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10229,7 +10229,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10251,7 +10251,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10273,7 +10273,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10295,7 +10295,7 @@
         <v>5.0500000000000003E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10317,29 +10317,29 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
       </c>
-      <c r="B81" s="17" t="str">
+      <c r="B81" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I82</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C81" s="47" t="str">
+        <v>4.2299999999999997E-2</v>
+      </c>
+      <c r="C81" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J82</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D81" s="47" t="str">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="D81" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K82</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E81" s="5" t="str">
+        <v>4.7800000000000002E-2</v>
+      </c>
+      <c r="E81" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L82</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.04E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10361,7 +10361,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10383,7 +10383,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10405,7 +10405,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10427,7 +10427,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10449,7 +10449,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10471,7 +10471,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10493,7 +10493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10515,7 +10515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10537,7 +10537,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10559,7 +10559,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10581,7 +10581,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10603,7 +10603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10625,7 +10625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10647,7 +10647,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10669,7 +10669,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10691,7 +10691,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10713,7 +10713,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10735,7 +10735,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10757,7 +10757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10779,7 +10779,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10801,7 +10801,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10823,7 +10823,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10845,7 +10845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10867,7 +10867,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10889,7 +10889,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10911,7 +10911,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10933,7 +10933,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10955,7 +10955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10977,7 +10977,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10999,7 +10999,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11021,7 +11021,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11043,7 +11043,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11065,7 +11065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11087,7 +11087,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11109,7 +11109,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11131,7 +11131,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11153,7 +11153,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11175,7 +11175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11197,7 +11197,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11219,7 +11219,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11241,7 +11241,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11263,7 +11263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11285,7 +11285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11307,7 +11307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11329,7 +11329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11351,7 +11351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11373,7 +11373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11395,7 +11395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11417,7 +11417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11439,7 +11439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11461,7 +11461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11483,7 +11483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11505,7 +11505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11527,7 +11527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11549,7 +11549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11571,7 +11571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11593,7 +11593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11615,7 +11615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11637,7 +11637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11659,7 +11659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11681,7 +11681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11703,7 +11703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11725,7 +11725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11747,7 +11747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11769,7 +11769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11791,7 +11791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11813,7 +11813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11835,7 +11835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11857,7 +11857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11879,7 +11879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11901,7 +11901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11923,7 +11923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11945,7 +11945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11967,7 +11967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11989,7 +11989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12011,7 +12011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12033,7 +12033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12055,7 +12055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12077,7 +12077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12099,7 +12099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12121,7 +12121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12143,7 +12143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12165,7 +12165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12187,7 +12187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12209,7 +12209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12231,7 +12231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12253,7 +12253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12275,7 +12275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12297,7 +12297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12319,7 +12319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12341,7 +12341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12363,7 +12363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12385,7 +12385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12407,7 +12407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12429,7 +12429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12451,7 +12451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12473,7 +12473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12495,7 +12495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12517,7 +12517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12539,7 +12539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12561,7 +12561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12583,7 +12583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12605,7 +12605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12627,7 +12627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12649,7 +12649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12671,7 +12671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12693,7 +12693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12715,7 +12715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12737,7 +12737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12759,7 +12759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12781,7 +12781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12803,7 +12803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12825,7 +12825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12847,7 +12847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12869,7 +12869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12891,7 +12891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12913,7 +12913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12935,7 +12935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12957,7 +12957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12979,7 +12979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13001,7 +13001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13023,7 +13023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13045,7 +13045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13067,7 +13067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13089,7 +13089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13111,7 +13111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13133,7 +13133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13155,7 +13155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13177,7 +13177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13199,7 +13199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13221,7 +13221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13243,7 +13243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13265,7 +13265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13287,7 +13287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13309,7 +13309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13331,7 +13331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13353,7 +13353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13375,7 +13375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13397,7 +13397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13419,7 +13419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13441,7 +13441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13463,7 +13463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13485,7 +13485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13507,7 +13507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13529,7 +13529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13551,7 +13551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13573,7 +13573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13595,7 +13595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13617,7 +13617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13639,7 +13639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13661,7 +13661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13683,7 +13683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13705,7 +13705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13727,7 +13727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13749,7 +13749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13771,7 +13771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13793,7 +13793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13815,7 +13815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13837,7 +13837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13859,7 +13859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13881,7 +13881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13903,7 +13903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13925,7 +13925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13947,7 +13947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13969,7 +13969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13991,7 +13991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14013,7 +14013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14035,7 +14035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14057,7 +14057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14079,7 +14079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14101,7 +14101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14123,7 +14123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14145,7 +14145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14167,7 +14167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14189,7 +14189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14211,7 +14211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14233,7 +14233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14255,7 +14255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14277,7 +14277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14299,7 +14299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14321,7 +14321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14343,7 +14343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14365,7 +14365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14387,7 +14387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14409,7 +14409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14431,7 +14431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14453,7 +14453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14475,7 +14475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14497,7 +14497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14519,7 +14519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14541,7 +14541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14563,7 +14563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14585,7 +14585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14607,7 +14607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14629,7 +14629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14651,7 +14651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14673,7 +14673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14695,7 +14695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14717,7 +14717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14739,7 +14739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14761,7 +14761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14783,7 +14783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14805,7 +14805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14827,7 +14827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14849,7 +14849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14871,7 +14871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14893,7 +14893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14915,7 +14915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14937,7 +14937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14959,7 +14959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14981,7 +14981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15003,7 +15003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15025,7 +15025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15047,7 +15047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15069,7 +15069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15091,7 +15091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15113,7 +15113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15135,7 +15135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15157,7 +15157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15179,7 +15179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15201,7 +15201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15223,7 +15223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15245,7 +15245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15267,7 +15267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15289,7 +15289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15311,7 +15311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15333,7 +15333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15355,7 +15355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15377,7 +15377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15399,7 +15399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15421,7 +15421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15443,7 +15443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15465,7 +15465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15487,7 +15487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15509,7 +15509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15531,7 +15531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15553,7 +15553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15575,7 +15575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15597,7 +15597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15619,7 +15619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15641,7 +15641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15663,7 +15663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15685,7 +15685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15707,7 +15707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15729,7 +15729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15751,7 +15751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15773,7 +15773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15795,7 +15795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15817,7 +15817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15839,7 +15839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15861,7 +15861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15883,7 +15883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15905,7 +15905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15927,7 +15927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15949,7 +15949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15971,7 +15971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15993,7 +15993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16015,7 +16015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16037,7 +16037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16059,7 +16059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16081,7 +16081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16103,7 +16103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16125,7 +16125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16147,7 +16147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16169,7 +16169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16191,7 +16191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16213,7 +16213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16235,7 +16235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16257,7 +16257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16279,7 +16279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16301,7 +16301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16323,7 +16323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16345,7 +16345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16367,7 +16367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16389,7 +16389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16411,7 +16411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16433,7 +16433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16455,7 +16455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16477,7 +16477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16499,7 +16499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16521,7 +16521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16543,7 +16543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16565,7 +16565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16587,7 +16587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16609,7 +16609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16631,7 +16631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16653,7 +16653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16675,37 +16675,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16721,13 +16721,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.42578125" customWidth="1"/>
+    <col min="2" max="5" width="13.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16736,14 +16736,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16752,7 +16752,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16761,7 +16761,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16778,7 +16778,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16800,7 +16800,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16822,7 +16822,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16844,7 +16844,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16866,7 +16866,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16883,13 +16883,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16898,7 +16898,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16907,12 +16907,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16921,7 +16921,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16938,7 +16938,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16962,7 +16962,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16986,7 +16986,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17010,7 +17010,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17034,7 +17034,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17042,7 +17042,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17050,7 +17050,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17060,7 +17060,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17070,7 +17070,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17088,7 +17088,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17110,7 +17110,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17132,7 +17132,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17154,7 +17154,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17184,7 +17184,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17192,7 +17192,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17202,7 +17202,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17212,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17228,7 +17228,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17248,7 +17248,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17268,7 +17268,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17288,7 +17288,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17308,7 +17308,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17317,7 +17317,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17328,7 +17328,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17339,7 +17339,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17362,7 +17362,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17397,7 +17397,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17432,7 +17432,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17467,7 +17467,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17519,193 +17519,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A1" s="65" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="63"/>
-      <c r="M1" s="61" t="str" cm="1">
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="67"/>
+      <c r="M1" s="65" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="63"/>
-      <c r="Y1" s="61" t="str" cm="1">
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="66"/>
+      <c r="W1" s="67"/>
+      <c r="Y1" s="65" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="62"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="62"/>
-      <c r="AC1" s="62"/>
-      <c r="AD1" s="62"/>
-      <c r="AE1" s="62"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="62"/>
-      <c r="AH1" s="62"/>
-      <c r="AI1" s="63"/>
-      <c r="AK1" s="61" t="str" cm="1">
+      <c r="Z1" s="66"/>
+      <c r="AA1" s="66"/>
+      <c r="AB1" s="66"/>
+      <c r="AC1" s="66"/>
+      <c r="AD1" s="66"/>
+      <c r="AE1" s="66"/>
+      <c r="AF1" s="66"/>
+      <c r="AG1" s="66"/>
+      <c r="AH1" s="66"/>
+      <c r="AI1" s="67"/>
+      <c r="AK1" s="65" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="62"/>
-      <c r="AM1" s="62"/>
-      <c r="AN1" s="62"/>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="62"/>
-      <c r="AS1" s="62"/>
-      <c r="AT1" s="62"/>
-      <c r="AU1" s="63"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
-      <c r="A2" s="64" t="str">
+      <c r="AL1" s="66"/>
+      <c r="AM1" s="66"/>
+      <c r="AN1" s="66"/>
+      <c r="AO1" s="66"/>
+      <c r="AP1" s="66"/>
+      <c r="AQ1" s="66"/>
+      <c r="AR1" s="66"/>
+      <c r="AS1" s="66"/>
+      <c r="AT1" s="66"/>
+      <c r="AU1" s="67"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="66"/>
-      <c r="M2" s="64" t="str">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="63"/>
+      <c r="M2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
-      <c r="V2" s="65"/>
-      <c r="W2" s="66"/>
-      <c r="Y2" s="64" t="str">
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="63"/>
+      <c r="Y2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="65"/>
-      <c r="AA2" s="65"/>
-      <c r="AB2" s="65"/>
-      <c r="AC2" s="65"/>
-      <c r="AD2" s="65"/>
-      <c r="AE2" s="65"/>
-      <c r="AF2" s="65"/>
-      <c r="AG2" s="65"/>
-      <c r="AH2" s="65"/>
-      <c r="AI2" s="66"/>
-      <c r="AK2" s="64" t="str">
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+      <c r="AE2" s="62"/>
+      <c r="AF2" s="62"/>
+      <c r="AG2" s="62"/>
+      <c r="AH2" s="62"/>
+      <c r="AI2" s="63"/>
+      <c r="AK2" s="61" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="65"/>
-      <c r="AM2" s="65"/>
-      <c r="AN2" s="65"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="65"/>
-      <c r="AS2" s="65"/>
-      <c r="AT2" s="65"/>
-      <c r="AU2" s="66"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AL2" s="62"/>
+      <c r="AM2" s="62"/>
+      <c r="AN2" s="62"/>
+      <c r="AO2" s="62"/>
+      <c r="AP2" s="62"/>
+      <c r="AQ2" s="62"/>
+      <c r="AR2" s="62"/>
+      <c r="AS2" s="62"/>
+      <c r="AT2" s="62"/>
+      <c r="AU2" s="63"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="67" t="s">
+      <c r="B3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="67"/>
-      <c r="D3" s="67"/>
-      <c r="E3" s="67"/>
-      <c r="F3" s="67"/>
-      <c r="G3" s="67"/>
-      <c r="H3" s="67"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="67"/>
-      <c r="K3" s="67"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="67" t="s">
+      <c r="N3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="67"/>
-      <c r="P3" s="67"/>
-      <c r="Q3" s="67"/>
-      <c r="R3" s="67"/>
-      <c r="S3" s="67"/>
-      <c r="T3" s="67"/>
-      <c r="U3" s="67"/>
-      <c r="V3" s="67"/>
-      <c r="W3" s="67"/>
+      <c r="O3" s="64"/>
+      <c r="P3" s="64"/>
+      <c r="Q3" s="64"/>
+      <c r="R3" s="64"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="64"/>
+      <c r="U3" s="64"/>
+      <c r="V3" s="64"/>
+      <c r="W3" s="64"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="67" t="s">
+      <c r="Z3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="67"/>
-      <c r="AE3" s="67"/>
-      <c r="AF3" s="67"/>
-      <c r="AG3" s="67"/>
-      <c r="AH3" s="67"/>
-      <c r="AI3" s="67"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
+      <c r="AG3" s="64"/>
+      <c r="AH3" s="64"/>
+      <c r="AI3" s="64"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="67" t="s">
+      <c r="AL3" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="67"/>
-      <c r="AN3" s="67"/>
-      <c r="AO3" s="67"/>
-      <c r="AP3" s="67"/>
-      <c r="AQ3" s="67"/>
-      <c r="AR3" s="67"/>
-      <c r="AS3" s="67"/>
-      <c r="AT3" s="67"/>
-      <c r="AU3" s="67"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17875,7 +17875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18009,7 +18009,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18183,7 +18183,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18357,7 +18357,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18531,7 +18531,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18705,7 +18705,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18879,7 +18879,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19053,7 +19053,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19227,7 +19227,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19401,7 +19401,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19575,7 +19575,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19749,7 +19749,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19923,7 +19923,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20097,7 +20097,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20271,7 +20271,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20445,7 +20445,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20619,7 +20619,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20793,7 +20793,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20967,7 +20967,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21141,7 +21141,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21315,7 +21315,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21489,7 +21489,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21663,7 +21663,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21837,7 +21837,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22011,7 +22011,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22185,7 +22185,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22359,7 +22359,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22533,7 +22533,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22707,7 +22707,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22881,7 +22881,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23055,7 +23055,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23229,7 +23229,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23405,18 +23405,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="AK1:AU1"/>
+    <mergeCell ref="AK2:AU2"/>
+    <mergeCell ref="AL3:AU3"/>
+    <mergeCell ref="Y1:AI1"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="Z3:AI3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="M1:W1"/>
     <mergeCell ref="M2:W2"/>
     <mergeCell ref="N3:W3"/>
-    <mergeCell ref="AK1:AU1"/>
-    <mergeCell ref="AK2:AU2"/>
-    <mergeCell ref="AL3:AU3"/>
-    <mergeCell ref="Y1:AI1"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="Z3:AI3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23429,7 +23429,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23450,7 +23450,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>333375</xdr:colOff>
+                <xdr:colOff>336550</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-21
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA7BFF2-3523-4C0C-8630-E9018763D16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BFE791-D15E-4929-93FD-BA8D734DAB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17565" yWindow="1110" windowWidth="12480" windowHeight="7770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45465" yWindow="1290" windowWidth="11055" windowHeight="7770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,6 +573,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -583,15 +592,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>336550</xdr:colOff>
+          <xdr:colOff>333375</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3372,17 +3372,17 @@
           <cell r="H83">
             <v>46101</v>
           </cell>
-          <cell r="I83" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J83" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K83" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L83" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I83">
+            <v>4.24E-2</v>
+          </cell>
+          <cell r="J83">
+            <v>4.5400000000000003E-2</v>
+          </cell>
+          <cell r="K83">
+            <v>4.7699999999999999E-2</v>
+          </cell>
+          <cell r="L83">
+            <v>5.0200000000000002E-2</v>
           </cell>
         </row>
         <row r="84">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,9 +8346,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8381,9 +8398,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8579,16 +8613,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8597,7 +8631,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8606,7 +8640,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8645,7 +8679,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8667,7 +8701,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8689,7 +8723,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8711,7 +8745,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8733,7 +8767,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8755,7 +8789,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8777,7 +8811,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8799,7 +8833,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8821,7 +8855,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8843,7 +8877,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8865,7 +8899,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8887,7 +8921,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8909,7 +8943,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8931,7 +8965,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8953,7 +8987,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -8975,7 +9009,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -8997,7 +9031,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9019,7 +9053,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9041,7 +9075,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9063,7 +9097,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9085,7 +9119,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9107,7 +9141,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9129,7 +9163,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9151,7 +9185,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9173,7 +9207,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9195,7 +9229,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9217,7 +9251,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9239,7 +9273,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9261,7 +9295,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9283,7 +9317,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9305,7 +9339,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9327,7 +9361,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9349,7 +9383,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9371,7 +9405,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9393,7 +9427,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9415,7 +9449,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9437,7 +9471,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9459,7 +9493,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9481,7 +9515,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9503,7 +9537,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9525,7 +9559,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9547,7 +9581,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9569,7 +9603,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9591,7 +9625,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9613,7 +9647,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9635,7 +9669,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9657,7 +9691,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9679,7 +9713,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9701,7 +9735,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9723,7 +9757,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9745,7 +9779,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9767,7 +9801,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9789,7 +9823,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9811,7 +9845,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9833,7 +9867,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9855,7 +9889,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9877,7 +9911,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9899,7 +9933,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9921,7 +9955,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9943,7 +9977,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9965,7 +9999,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -9987,7 +10021,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10009,7 +10043,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10031,7 +10065,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10053,7 +10087,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10075,7 +10109,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10097,7 +10131,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10119,7 +10153,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10141,7 +10175,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10163,7 +10197,7 @@
         <v>4.9099999999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10185,7 +10219,7 @@
         <v>5.0099999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10207,7 +10241,7 @@
         <v>5.0700000000000002E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10229,7 +10263,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10251,7 +10285,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10273,7 +10307,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10295,7 +10329,7 @@
         <v>5.0500000000000003E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10317,7 +10351,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10339,29 +10373,29 @@
         <v>5.04E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
       </c>
-      <c r="B82" s="17" t="str">
+      <c r="B82" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I83</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C82" s="47" t="str">
+        <v>4.24E-2</v>
+      </c>
+      <c r="C82" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J83</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D82" s="47" t="str">
+        <v>4.5400000000000003E-2</v>
+      </c>
+      <c r="D82" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K83</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E82" s="5" t="str">
+        <v>4.7699999999999999E-2</v>
+      </c>
+      <c r="E82" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L83</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+        <v>5.0200000000000002E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
@@ -10383,7 +10417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
@@ -10405,7 +10439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
@@ -10427,7 +10461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10449,7 +10483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10471,7 +10505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10493,7 +10527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10515,7 +10549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10537,7 +10571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10559,7 +10593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10581,7 +10615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10603,7 +10637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10625,7 +10659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10647,7 +10681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10669,7 +10703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10691,7 +10725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10713,7 +10747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10735,7 +10769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10757,7 +10791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10779,7 +10813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10801,7 +10835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10823,7 +10857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10845,7 +10879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10867,7 +10901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10889,7 +10923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10911,7 +10945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10933,7 +10967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10955,7 +10989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -10977,7 +11011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -10999,7 +11033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11021,7 +11055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11043,7 +11077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11065,7 +11099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11087,7 +11121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11109,7 +11143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11131,7 +11165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11153,7 +11187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11175,7 +11209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11197,7 +11231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11219,7 +11253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11241,7 +11275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11263,7 +11297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11285,7 +11319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11307,7 +11341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11329,7 +11363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11351,7 +11385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11373,7 +11407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11395,7 +11429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11417,7 +11451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11439,7 +11473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11461,7 +11495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11483,7 +11517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11505,7 +11539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11527,7 +11561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11549,7 +11583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11571,7 +11605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11593,7 +11627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11615,7 +11649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11637,7 +11671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11659,7 +11693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11681,7 +11715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11703,7 +11737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11725,7 +11759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11747,7 +11781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11769,7 +11803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11791,7 +11825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11813,7 +11847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11835,7 +11869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11857,7 +11891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11879,7 +11913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11901,7 +11935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11923,7 +11957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11945,7 +11979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -11967,7 +12001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -11989,7 +12023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12011,7 +12045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12033,7 +12067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12055,7 +12089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12077,7 +12111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12099,7 +12133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12121,7 +12155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12143,7 +12177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12165,7 +12199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12187,7 +12221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12209,7 +12243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12231,7 +12265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12253,7 +12287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12275,7 +12309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12297,7 +12331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12319,7 +12353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12341,7 +12375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12363,7 +12397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12385,7 +12419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12407,7 +12441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12429,7 +12463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12451,7 +12485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12473,7 +12507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12495,7 +12529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12517,7 +12551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12539,7 +12573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12561,7 +12595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12583,7 +12617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12605,7 +12639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12627,7 +12661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12649,7 +12683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12671,7 +12705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12693,7 +12727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12715,7 +12749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12737,7 +12771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12759,7 +12793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12781,7 +12815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12803,7 +12837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12825,7 +12859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12847,7 +12881,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12869,7 +12903,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12891,7 +12925,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12913,7 +12947,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12935,7 +12969,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12957,7 +12991,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -12979,7 +13013,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13001,7 +13035,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13023,7 +13057,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13045,7 +13079,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13067,7 +13101,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13089,7 +13123,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13111,7 +13145,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13133,7 +13167,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13155,7 +13189,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13177,7 +13211,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13199,7 +13233,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13221,7 +13255,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13243,7 +13277,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13265,7 +13299,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13287,7 +13321,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13309,7 +13343,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13331,7 +13365,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13353,7 +13387,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13375,7 +13409,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13397,7 +13431,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13419,7 +13453,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13441,7 +13475,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13463,7 +13497,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13485,7 +13519,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13507,7 +13541,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13529,7 +13563,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13551,7 +13585,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13573,7 +13607,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13595,7 +13629,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13617,7 +13651,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13639,7 +13673,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13661,7 +13695,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13683,7 +13717,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13705,7 +13739,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13727,7 +13761,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13749,7 +13783,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13771,7 +13805,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13793,7 +13827,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13815,7 +13849,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13837,7 +13871,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13859,7 +13893,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H243</f>
         <v>46261</v>
@@ -13881,7 +13915,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H244</f>
         <v>46262</v>
@@ -13903,7 +13937,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H245</f>
         <v>46263</v>
@@ -13925,7 +13959,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H246</f>
         <v>46264</v>
@@ -13947,7 +13981,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H247</f>
         <v>46265</v>
@@ -13969,7 +14003,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H248</f>
         <v>46266</v>
@@ -13991,7 +14025,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H249</f>
         <v>46267</v>
@@ -14013,7 +14047,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H250</f>
         <v>46268</v>
@@ -14035,7 +14069,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H251</f>
         <v>46269</v>
@@ -14057,7 +14091,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H252</f>
         <v>46270</v>
@@ -14079,7 +14113,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H253</f>
         <v>46271</v>
@@ -14101,7 +14135,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H254</f>
         <v>46272</v>
@@ -14123,7 +14157,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H255</f>
         <v>46273</v>
@@ -14145,7 +14179,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H256</f>
         <v>46274</v>
@@ -14167,7 +14201,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H257</f>
         <v>46275</v>
@@ -14189,7 +14223,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H258</f>
         <v>46276</v>
@@ -14211,7 +14245,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H259</f>
         <v>46277</v>
@@ -14233,7 +14267,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H260</f>
         <v>46278</v>
@@ -14255,7 +14289,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H261</f>
         <v>46279</v>
@@ -14277,7 +14311,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H262</f>
         <v>46280</v>
@@ -14299,7 +14333,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H263</f>
         <v>46281</v>
@@ -14321,7 +14355,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H264</f>
         <v>46282</v>
@@ -14343,7 +14377,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H265</f>
         <v>46283</v>
@@ -14365,7 +14399,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H266</f>
         <v>46284</v>
@@ -14387,7 +14421,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H267</f>
         <v>46285</v>
@@ -14409,7 +14443,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H268</f>
         <v>46286</v>
@@ -14431,7 +14465,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H269</f>
         <v>46287</v>
@@ -14453,7 +14487,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H270</f>
         <v>46288</v>
@@ -14475,7 +14509,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H271</f>
         <v>46289</v>
@@ -14497,7 +14531,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H272</f>
         <v>46290</v>
@@ -14519,7 +14553,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H273</f>
         <v>46291</v>
@@ -14541,7 +14575,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H274</f>
         <v>46292</v>
@@ -14563,7 +14597,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H275</f>
         <v>46293</v>
@@ -14585,7 +14619,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H276</f>
         <v>46294</v>
@@ -14607,7 +14641,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H277</f>
         <v>46295</v>
@@ -14629,7 +14663,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H278</f>
         <v>46296</v>
@@ -14651,7 +14685,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H279</f>
         <v>46297</v>
@@ -14673,7 +14707,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H280</f>
         <v>46298</v>
@@ -14695,7 +14729,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H281</f>
         <v>46299</v>
@@ -14717,7 +14751,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H282</f>
         <v>46300</v>
@@ -14739,7 +14773,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H283</f>
         <v>46301</v>
@@ -14761,7 +14795,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H284</f>
         <v>46302</v>
@@ -14783,7 +14817,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H285</f>
         <v>46303</v>
@@ -14805,7 +14839,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H286</f>
         <v>46304</v>
@@ -14827,7 +14861,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H287</f>
         <v>46305</v>
@@ -14849,7 +14883,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H288</f>
         <v>46306</v>
@@ -14871,7 +14905,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H289</f>
         <v>46307</v>
@@ -14893,7 +14927,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H290</f>
         <v>46308</v>
@@ -14915,7 +14949,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H291</f>
         <v>46309</v>
@@ -14937,7 +14971,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H292</f>
         <v>46310</v>
@@ -14959,7 +14993,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H293</f>
         <v>46311</v>
@@ -14981,7 +15015,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H294</f>
         <v>46312</v>
@@ -15003,7 +15037,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H295</f>
         <v>46313</v>
@@ -15025,7 +15059,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H296</f>
         <v>46314</v>
@@ -15047,7 +15081,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H297</f>
         <v>46315</v>
@@ -15069,7 +15103,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H298</f>
         <v>46316</v>
@@ -15091,7 +15125,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H299</f>
         <v>46317</v>
@@ -15113,7 +15147,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H300</f>
         <v>46318</v>
@@ -15135,7 +15169,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H301</f>
         <v>46319</v>
@@ -15157,7 +15191,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H302</f>
         <v>46320</v>
@@ -15179,7 +15213,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H303</f>
         <v>46321</v>
@@ -15201,7 +15235,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H304</f>
         <v>46322</v>
@@ -15223,7 +15257,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H305</f>
         <v>46323</v>
@@ -15245,7 +15279,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H306</f>
         <v>46324</v>
@@ -15267,7 +15301,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H307</f>
         <v>46325</v>
@@ -15289,7 +15323,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H308</f>
         <v>46326</v>
@@ -15311,7 +15345,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H309</f>
         <v>46327</v>
@@ -15333,7 +15367,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H310</f>
         <v>46328</v>
@@ -15355,7 +15389,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H311</f>
         <v>46329</v>
@@ -15377,7 +15411,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H312</f>
         <v>46330</v>
@@ -15399,7 +15433,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H313</f>
         <v>46331</v>
@@ -15421,7 +15455,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H314</f>
         <v>46332</v>
@@ -15443,7 +15477,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H315</f>
         <v>46333</v>
@@ -15465,7 +15499,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H316</f>
         <v>46334</v>
@@ -15487,7 +15521,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H317</f>
         <v>46335</v>
@@ -15509,7 +15543,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H318</f>
         <v>46336</v>
@@ -15531,7 +15565,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H319</f>
         <v>46337</v>
@@ -15553,7 +15587,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H320</f>
         <v>46338</v>
@@ -15575,7 +15609,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H321</f>
         <v>46339</v>
@@ -15597,7 +15631,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H322</f>
         <v>46340</v>
@@ -15619,7 +15653,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H323</f>
         <v>46341</v>
@@ -15641,7 +15675,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H324</f>
         <v>46342</v>
@@ -15663,7 +15697,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H325</f>
         <v>46343</v>
@@ -15685,7 +15719,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H326</f>
         <v>46344</v>
@@ -15707,7 +15741,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H327</f>
         <v>46345</v>
@@ -15729,7 +15763,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H328</f>
         <v>46346</v>
@@ -15751,7 +15785,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H329</f>
         <v>46347</v>
@@ -15773,7 +15807,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H330</f>
         <v>46348</v>
@@ -15795,7 +15829,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H331</f>
         <v>46349</v>
@@ -15817,7 +15851,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H332</f>
         <v>46350</v>
@@ -15839,7 +15873,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H333</f>
         <v>46351</v>
@@ -15861,7 +15895,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H334</f>
         <v>46352</v>
@@ -15883,7 +15917,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H335</f>
         <v>46353</v>
@@ -15905,7 +15939,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H336</f>
         <v>46354</v>
@@ -15927,7 +15961,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H337</f>
         <v>46355</v>
@@ -15949,7 +15983,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H338</f>
         <v>46356</v>
@@ -15971,7 +16005,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H339</f>
         <v>46357</v>
@@ -15993,7 +16027,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H340</f>
         <v>46358</v>
@@ -16015,7 +16049,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H341</f>
         <v>46359</v>
@@ -16037,7 +16071,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H342</f>
         <v>46360</v>
@@ -16059,7 +16093,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H343</f>
         <v>46361</v>
@@ -16081,7 +16115,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H344</f>
         <v>46362</v>
@@ -16103,7 +16137,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H345</f>
         <v>46363</v>
@@ -16125,7 +16159,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H346</f>
         <v>46364</v>
@@ -16147,7 +16181,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H347</f>
         <v>46365</v>
@@ -16169,7 +16203,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H348</f>
         <v>46366</v>
@@ -16191,7 +16225,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H349</f>
         <v>46367</v>
@@ -16213,7 +16247,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H350</f>
         <v>46368</v>
@@ -16235,7 +16269,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H351</f>
         <v>46369</v>
@@ -16257,7 +16291,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H352</f>
         <v>46370</v>
@@ -16279,7 +16313,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H353</f>
         <v>46371</v>
@@ -16301,7 +16335,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H354</f>
         <v>46372</v>
@@ -16323,7 +16357,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H355</f>
         <v>46373</v>
@@ -16345,7 +16379,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H356</f>
         <v>46374</v>
@@ -16367,7 +16401,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H357</f>
         <v>46375</v>
@@ -16389,7 +16423,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H358</f>
         <v>46376</v>
@@ -16411,7 +16445,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H359</f>
         <v>46377</v>
@@ -16433,7 +16467,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H360</f>
         <v>46378</v>
@@ -16455,7 +16489,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H361</f>
         <v>46379</v>
@@ -16477,7 +16511,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H362</f>
         <v>46380</v>
@@ -16499,7 +16533,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H363</f>
         <v>46381</v>
@@ -16521,7 +16555,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H364</f>
         <v>46382</v>
@@ -16543,7 +16577,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H365</f>
         <v>46383</v>
@@ -16565,7 +16599,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H366</f>
         <v>46384</v>
@@ -16587,7 +16621,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H367</f>
         <v>46385</v>
@@ -16609,7 +16643,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H368</f>
         <v>46386</v>
@@ -16631,7 +16665,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H369</f>
         <v>46387</v>
@@ -16653,7 +16687,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" s="45">
         <f>'[1]Jumbo Bus Date to PDD'!H370</f>
         <v>46388</v>
@@ -16675,37 +16709,37 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" s="15"/>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" s="15"/>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" s="15"/>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" s="15"/>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" s="15"/>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" s="15"/>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" s="15"/>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" s="15"/>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" s="15"/>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" s="15"/>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" s="15"/>
     </row>
   </sheetData>
@@ -16721,13 +16755,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="5" width="13.453125" customWidth="1"/>
+    <col min="2" max="5" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="54" t="s">
         <v>8</v>
       </c>
@@ -16736,14 +16770,14 @@
       <c r="D1" s="55"/>
       <c r="E1" s="56"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="51" t="s">
         <v>5</v>
@@ -16752,7 +16786,7 @@
       <c r="D3" s="52"/>
       <c r="E3" s="53"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>6</v>
       </c>
@@ -16761,7 +16795,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>7</v>
       </c>
@@ -16778,7 +16812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")</f>
         <v>1/1/2026 - 3/31/2026</v>
@@ -16800,7 +16834,7 @@
         <v>4.7500000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")</f>
         <v>4/1/2026 - 6/30/2026</v>
@@ -16822,7 +16856,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")</f>
         <v>7/1/2026 - 9/30/2026</v>
@@ -16844,7 +16878,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,10,1),"m/d/yyyy") &amp;" - " &amp;TEXT(DATE([1]!Year_of_Valuation,12,31),"m/d/yyyy")</f>
         <v>10/1/2026 - 12/31/2026</v>
@@ -16866,7 +16900,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="48"/>
     </row>
   </sheetData>
@@ -16883,13 +16917,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="7" width="16" customWidth="1"/>
-    <col min="8" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="60" t="s">
         <v>41</v>
       </c>
@@ -16898,7 +16932,7 @@
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="60" t="s">
         <v>42</v>
       </c>
@@ -16907,12 +16941,12 @@
       <c r="D2" s="60"/>
       <c r="E2" s="60"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="51" t="s">
         <v>9</v>
       </c>
@@ -16921,7 +16955,7 @@
       <c r="D4" s="52"/>
       <c r="E4" s="53"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>10</v>
       </c>
@@ -16938,7 +16972,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>0</v>
       </c>
@@ -16962,7 +16996,7 @@
       <c r="H6" s="22"/>
       <c r="I6" s="22"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>1</v>
       </c>
@@ -16986,7 +17020,7 @@
       <c r="H7" s="22"/>
       <c r="I7" s="22"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>2</v>
       </c>
@@ -17010,7 +17044,7 @@
       <c r="H8" s="22"/>
       <c r="I8" s="22"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
@@ -17034,7 +17068,7 @@
       <c r="H9" s="22"/>
       <c r="I9" s="22"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -17042,7 +17076,7 @@
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22"/>
       <c r="C11" s="22"/>
@@ -17050,7 +17084,7 @@
       <c r="E11" s="22"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -17060,7 +17094,7 @@
       <c r="E12" s="22"/>
       <c r="F12" s="22"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="57" t="s">
         <v>9</v>
       </c>
@@ -17070,7 +17104,7 @@
       <c r="E13" s="59"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>10</v>
       </c>
@@ -17088,7 +17122,7 @@
       </c>
       <c r="F14" s="22"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
@@ -17110,7 +17144,7 @@
       </c>
       <c r="F15" s="22"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>1</v>
       </c>
@@ -17132,7 +17166,7 @@
       </c>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>2</v>
       </c>
@@ -17154,7 +17188,7 @@
       </c>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
@@ -17176,7 +17210,7 @@
       </c>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
@@ -17184,7 +17218,7 @@
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
@@ -17192,7 +17226,7 @@
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -17202,7 +17236,7 @@
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="57" t="s">
         <v>9</v>
       </c>
@@ -17212,7 +17246,7 @@
       <c r="E22" s="22"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>10</v>
       </c>
@@ -17228,7 +17262,7 @@
       <c r="E23" s="27"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="28" t="s">
         <v>0</v>
       </c>
@@ -17248,7 +17282,7 @@
       <c r="F24" s="22"/>
       <c r="H24" s="22"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
         <v>1</v>
       </c>
@@ -17268,7 +17302,7 @@
       <c r="F25" s="22"/>
       <c r="H25" s="22"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
         <v>2</v>
       </c>
@@ -17288,7 +17322,7 @@
       <c r="F26" s="22"/>
       <c r="H26" s="22"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
         <v>3</v>
       </c>
@@ -17308,7 +17342,7 @@
       <c r="F27" s="22"/>
       <c r="H27" s="22"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -17317,7 +17351,7 @@
       <c r="F28" s="22"/>
       <c r="G28" s="22"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -17328,7 +17362,7 @@
       <c r="F29" s="22"/>
       <c r="G29" s="22"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="57" t="s">
         <v>9</v>
       </c>
@@ -17339,7 +17373,7 @@
       <c r="F30" s="58"/>
       <c r="G30" s="59"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="26" t="s">
         <v>10</v>
       </c>
@@ -17362,7 +17396,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="28" t="s">
         <v>0</v>
       </c>
@@ -17397,7 +17431,7 @@
       <c r="L32" s="22"/>
       <c r="M32" s="22"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
         <v>21</v>
       </c>
@@ -17432,7 +17466,7 @@
       <c r="L33" s="22"/>
       <c r="M33" s="22"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
         <v>2</v>
       </c>
@@ -17467,7 +17501,7 @@
       <c r="L34" s="22"/>
       <c r="M34" s="22"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="23" t="s">
         <v>3</v>
       </c>
@@ -17519,193 +17553,193 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{960AAD26-B121-4BD5-9ACA-ACA8580C5ADA}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:AU36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="13" customWidth="1"/>
     <col min="37" max="37" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A1" s="65" t="str" cm="1">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A1" s="61" t="str" cm="1">
         <f t="array" ref="A1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q1 VM - V Table X"</f>
         <v>2026 Q1 VM - V Table X</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="67"/>
-      <c r="M1" s="65" t="str" cm="1">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="63"/>
+      <c r="M1" s="61" t="str" cm="1">
         <f t="array" ref="M1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q2 VM - 22 Table X"</f>
         <v>2026 Q2 VM - 22 Table X</v>
       </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="66"/>
-      <c r="U1" s="66"/>
-      <c r="V1" s="66"/>
-      <c r="W1" s="67"/>
-      <c r="Y1" s="65" t="str" cm="1">
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
+      <c r="T1" s="62"/>
+      <c r="U1" s="62"/>
+      <c r="V1" s="62"/>
+      <c r="W1" s="63"/>
+      <c r="Y1" s="61" t="str" cm="1">
         <f t="array" ref="Y1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q3 VM - 22 Table X"</f>
         <v>2026 Q3 VM - 22 Table X</v>
       </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="66"/>
-      <c r="AC1" s="66"/>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="66"/>
-      <c r="AG1" s="66"/>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="67"/>
-      <c r="AK1" s="65" t="str" cm="1">
+      <c r="Z1" s="62"/>
+      <c r="AA1" s="62"/>
+      <c r="AB1" s="62"/>
+      <c r="AC1" s="62"/>
+      <c r="AD1" s="62"/>
+      <c r="AE1" s="62"/>
+      <c r="AF1" s="62"/>
+      <c r="AG1" s="62"/>
+      <c r="AH1" s="62"/>
+      <c r="AI1" s="63"/>
+      <c r="AK1" s="61" t="str" cm="1">
         <f t="array" ref="AK1">TEXT([1]!Year_of_Valuation,"0000")&amp; " Q4 VM - 22 Table X"</f>
         <v>2026 Q4 VM - 22 Table X</v>
       </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="66"/>
-      <c r="AO1" s="66"/>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="66"/>
-      <c r="AS1" s="66"/>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="67"/>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
-      <c r="A2" s="61" t="str">
+      <c r="AL1" s="62"/>
+      <c r="AM1" s="62"/>
+      <c r="AN1" s="62"/>
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="62"/>
+      <c r="AS1" s="62"/>
+      <c r="AT1" s="62"/>
+      <c r="AU1" s="63"/>
+    </row>
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
+      <c r="A2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation-1,10,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation-1,12,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>10/1/2025 thru 12/31/2025 Quarterly Average Spread Data</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="63"/>
-      <c r="M2" s="61" t="str">
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="66"/>
+      <c r="M2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,1,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,3,31),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>1/1/2026 thru 3/31/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="63"/>
-      <c r="Y2" s="61" t="str">
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="65"/>
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="66"/>
+      <c r="Y2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,4,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,6,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>4/1/2026 thru 6/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="63"/>
-      <c r="AK2" s="61" t="str">
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="65"/>
+      <c r="AE2" s="65"/>
+      <c r="AF2" s="65"/>
+      <c r="AG2" s="65"/>
+      <c r="AH2" s="65"/>
+      <c r="AI2" s="66"/>
+      <c r="AK2" s="64" t="str">
         <f>TEXT(DATE([1]!Year_of_Valuation,7,1),"m/d/yyyy")&amp; " thru " &amp; TEXT(DATE([1]!Year_of_Valuation,9,30),"m/d/yyyy")&amp; " Quarterly Average Spread Data"</f>
         <v>7/1/2026 thru 9/30/2026 Quarterly Average Spread Data</v>
       </c>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="63"/>
-    </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AL2" s="65"/>
+      <c r="AM2" s="65"/>
+      <c r="AN2" s="65"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="65"/>
+      <c r="AS2" s="65"/>
+      <c r="AT2" s="65"/>
+      <c r="AU2" s="66"/>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
       <c r="M3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="64" t="s">
+      <c r="N3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+      <c r="Q3" s="67"/>
+      <c r="R3" s="67"/>
+      <c r="S3" s="67"/>
+      <c r="T3" s="67"/>
+      <c r="U3" s="67"/>
+      <c r="V3" s="67"/>
+      <c r="W3" s="67"/>
       <c r="Y3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="64" t="s">
+      <c r="Z3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
-      <c r="AD3" s="64"/>
-      <c r="AE3" s="64"/>
-      <c r="AF3" s="64"/>
-      <c r="AG3" s="64"/>
-      <c r="AH3" s="64"/>
-      <c r="AI3" s="64"/>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="67"/>
+      <c r="AE3" s="67"/>
+      <c r="AF3" s="67"/>
+      <c r="AG3" s="67"/>
+      <c r="AH3" s="67"/>
+      <c r="AI3" s="67"/>
       <c r="AK3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AL3" s="64" t="s">
+      <c r="AL3" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="AM3" s="64"/>
-      <c r="AN3" s="64"/>
-      <c r="AO3" s="64"/>
-      <c r="AP3" s="64"/>
-      <c r="AQ3" s="64"/>
-      <c r="AR3" s="64"/>
-      <c r="AS3" s="64"/>
-      <c r="AT3" s="64"/>
-      <c r="AU3" s="64"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+      <c r="AM3" s="67"/>
+      <c r="AN3" s="67"/>
+      <c r="AO3" s="67"/>
+      <c r="AP3" s="67"/>
+      <c r="AQ3" s="67"/>
+      <c r="AR3" s="67"/>
+      <c r="AS3" s="67"/>
+      <c r="AT3" s="67"/>
+      <c r="AU3" s="67"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
@@ -17875,7 +17909,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
@@ -18009,7 +18043,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" s="42">
         <v>1</v>
       </c>
@@ -18183,7 +18217,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A7" s="42">
         <v>2</v>
       </c>
@@ -18357,7 +18391,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" s="42">
         <v>3</v>
       </c>
@@ -18531,7 +18565,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A9" s="42">
         <v>4</v>
       </c>
@@ -18705,7 +18739,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A10" s="42">
         <v>5</v>
       </c>
@@ -18879,7 +18913,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A11" s="42">
         <v>6</v>
       </c>
@@ -19053,7 +19087,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A12" s="42">
         <v>7</v>
       </c>
@@ -19227,7 +19261,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" s="42">
         <v>8</v>
       </c>
@@ -19401,7 +19435,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" s="42">
         <v>9</v>
       </c>
@@ -19575,7 +19609,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" s="42">
         <v>10</v>
       </c>
@@ -19749,7 +19783,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A16" s="42">
         <v>11</v>
       </c>
@@ -19923,7 +19957,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A17" s="42">
         <v>12</v>
       </c>
@@ -20097,7 +20131,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A18" s="42">
         <v>13</v>
       </c>
@@ -20271,7 +20305,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A19" s="42">
         <v>14</v>
       </c>
@@ -20445,7 +20479,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" s="42">
         <v>15</v>
       </c>
@@ -20619,7 +20653,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="42">
         <v>16</v>
       </c>
@@ -20793,7 +20827,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A22" s="42">
         <v>17</v>
       </c>
@@ -20967,7 +21001,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A23" s="42">
         <v>18</v>
       </c>
@@ -21141,7 +21175,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="42">
         <v>19</v>
       </c>
@@ -21315,7 +21349,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A25" s="42">
         <v>20</v>
       </c>
@@ -21489,7 +21523,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" s="42">
         <v>21</v>
       </c>
@@ -21663,7 +21697,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A27" s="42">
         <v>22</v>
       </c>
@@ -21837,7 +21871,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A28" s="42">
         <v>23</v>
       </c>
@@ -22011,7 +22045,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A29" s="42">
         <v>24</v>
       </c>
@@ -22185,7 +22219,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A30" s="42">
         <v>25</v>
       </c>
@@ -22359,7 +22393,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" s="42">
         <v>26</v>
       </c>
@@ -22533,7 +22567,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" s="42">
         <v>27</v>
       </c>
@@ -22707,7 +22741,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A33" s="42">
         <v>28</v>
       </c>
@@ -22881,7 +22915,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A34" s="42">
         <v>29</v>
       </c>
@@ -23055,7 +23089,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A35" s="42">
         <v>30</v>
       </c>
@@ -23229,7 +23263,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A36" s="42" t="s">
         <v>36</v>
       </c>
@@ -23405,18 +23439,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="M2:W2"/>
+    <mergeCell ref="N3:W3"/>
     <mergeCell ref="AK1:AU1"/>
     <mergeCell ref="AK2:AU2"/>
     <mergeCell ref="AL3:AU3"/>
     <mergeCell ref="Y1:AI1"/>
     <mergeCell ref="Y2:AI2"/>
     <mergeCell ref="Z3:AI3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="M1:W1"/>
-    <mergeCell ref="M2:W2"/>
-    <mergeCell ref="N3:W3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -23429,7 +23463,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <sheetProtection algorithmName="SHA-512" hashValue="yvv3wbdeRzmlM4bzNOO2apq3mx/qVFX0Msifl9YhWgFuHibBrkknge+pGfxzSIcsAi5W1vdadtYqYf6xCYTqPg==" saltValue="d9XYKX9Q0BviUTprb1l8GA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23450,7 +23484,7 @@
               </from>
               <to>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>336550</xdr:colOff>
+                <xdr:colOff>333375</xdr:colOff>
                 <xdr:row>21</xdr:row>
                 <xdr:rowOff>171450</xdr:rowOff>
               </to>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-03-24
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
+++ b/docs/content_history/pbr-2026-vmv-nonjumbo-jumbo-valuation-rates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BFE791-D15E-4929-93FD-BA8D734DAB70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607B1BE5-7A46-4735-80C9-63600DA4CC9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="45465" yWindow="1290" windowWidth="11055" windowHeight="7770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Jumbo Rates" sheetId="4" r:id="rId1"/>
@@ -573,15 +573,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -592,6 +583,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -627,7 +627,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>11</xdr:col>
-          <xdr:colOff>333375</xdr:colOff>
+          <xdr:colOff>336550</xdr:colOff>
           <xdr:row>21</xdr:row>
           <xdr:rowOff>171450</xdr:rowOff>
         </xdr:to>
@@ -3389,51 +3389,51 @@
           <cell r="H84">
             <v>46102</v>
           </cell>
-          <cell r="I84" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J84" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K84" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L84" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I84">
+            <v>4.3400000000000001E-2</v>
+          </cell>
+          <cell r="J84">
+            <v>4.65E-2</v>
+          </cell>
+          <cell r="K84">
+            <v>4.9000000000000002E-2</v>
+          </cell>
+          <cell r="L84">
+            <v>5.1499999999999997E-2</v>
           </cell>
         </row>
         <row r="85">
           <cell r="H85">
             <v>46103</v>
           </cell>
-          <cell r="I85" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J85" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K85" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L85" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I85">
+            <v>4.3400000000000001E-2</v>
+          </cell>
+          <cell r="J85">
+            <v>4.65E-2</v>
+          </cell>
+          <cell r="K85">
+            <v>4.9000000000000002E-2</v>
+          </cell>
+          <cell r="L85">
+            <v>5.1499999999999997E-2</v>
           </cell>
         </row>
         <row r="86">
           <cell r="H86">
             <v>46104</v>
           </cell>
-          <cell r="I86" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="J86" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="K86" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
-          <cell r="L86" t="str">
-            <v xml:space="preserve"> </v>
+          <cell r="I86">
+            <v>4.3400000000000001E-2</v>
+          </cell>
+          <cell r="J86">
+            <v>4.65E-2</v>
+          </cell>
+          <cell r="K86">
+            <v>4.9000000000000002E-2</v>
+          </cell>
+          <cell r="L86">
+            <v>5.1499999999999997E-2</v>
           </cell>
         </row>
         <row r="87">
@@ -8271,9 +8271,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8311,9 +8311,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8346,26 +8346,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8398,26 +8381,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8613,16 +8579,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:E380"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="5" max="5" width="12.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="46"/>
       <c r="B1" s="51" t="s">
         <v>4</v>
@@ -8631,7 +8597,7 @@
       <c r="D1" s="52"/>
       <c r="E1" s="53"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
@@ -8640,7 +8606,7 @@
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>7</v>
       </c>
@@ -8657,7 +8623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H5</f>
         <v>46023</v>
@@ -8679,7 +8645,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H6</f>
         <v>46024</v>
@@ -8701,7 +8667,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H7</f>
         <v>46025</v>
@@ -8723,7 +8689,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H8</f>
         <v>46026</v>
@@ -8745,7 +8711,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H9</f>
         <v>46027</v>
@@ -8767,7 +8733,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H10</f>
         <v>46028</v>
@@ -8789,7 +8755,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H11</f>
         <v>46029</v>
@@ -8811,7 +8777,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H12</f>
         <v>46030</v>
@@ -8833,7 +8799,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H13</f>
         <v>46031</v>
@@ -8855,7 +8821,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H14</f>
         <v>46032</v>
@@ -8877,7 +8843,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H15</f>
         <v>46033</v>
@@ -8899,7 +8865,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H16</f>
         <v>46034</v>
@@ -8921,7 +8887,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H17</f>
         <v>46035</v>
@@ -8943,7 +8909,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H18</f>
         <v>46036</v>
@@ -8965,7 +8931,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H19</f>
         <v>46037</v>
@@ -8987,7 +8953,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H20</f>
         <v>46038</v>
@@ -9009,7 +8975,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H21</f>
         <v>46039</v>
@@ -9031,7 +8997,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H22</f>
         <v>46040</v>
@@ -9053,7 +9019,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H23</f>
         <v>46041</v>
@@ -9075,7 +9041,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H24</f>
         <v>46042</v>
@@ -9097,7 +9063,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H25</f>
         <v>46043</v>
@@ -9119,7 +9085,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H26</f>
         <v>46044</v>
@@ -9141,7 +9107,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H27</f>
         <v>46045</v>
@@ -9163,7 +9129,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H28</f>
         <v>46046</v>
@@ -9185,7 +9151,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H29</f>
         <v>46047</v>
@@ -9207,7 +9173,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H30</f>
         <v>46048</v>
@@ -9229,7 +9195,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H31</f>
         <v>46049</v>
@@ -9251,7 +9217,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H32</f>
         <v>46050</v>
@@ -9273,7 +9239,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H33</f>
         <v>46051</v>
@@ -9295,7 +9261,7 @@
         <v>4.8300000000000003E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H34</f>
         <v>46052</v>
@@ -9317,7 +9283,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H35</f>
         <v>46053</v>
@@ -9339,7 +9305,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H36</f>
         <v>46054</v>
@@ -9361,7 +9327,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H37</f>
         <v>46055</v>
@@ -9383,7 +9349,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H38</f>
         <v>46056</v>
@@ -9405,7 +9371,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H39</f>
         <v>46057</v>
@@ -9427,7 +9393,7 @@
         <v>4.8800000000000003E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H40</f>
         <v>46058</v>
@@ -9449,7 +9415,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H41</f>
         <v>46059</v>
@@ -9471,7 +9437,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H42</f>
         <v>46060</v>
@@ -9493,7 +9459,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H43</f>
         <v>46061</v>
@@ -9515,7 +9481,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H44</f>
         <v>46062</v>
@@ -9537,7 +9503,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H45</f>
         <v>46063</v>
@@ -9559,7 +9525,7 @@
         <v>4.8399999999999999E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H46</f>
         <v>46064</v>
@@ -9581,7 +9547,7 @@
         <v>4.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H47</f>
         <v>46065</v>
@@ -9603,7 +9569,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H48</f>
         <v>46066</v>
@@ -9625,7 +9591,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H49</f>
         <v>46067</v>
@@ -9647,7 +9613,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H50</f>
         <v>46068</v>
@@ -9669,7 +9635,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H51</f>
         <v>46069</v>
@@ -9691,7 +9657,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H52</f>
         <v>46070</v>
@@ -9713,7 +9679,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H53</f>
         <v>46071</v>
@@ -9735,7 +9701,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H54</f>
         <v>46072</v>
@@ -9757,7 +9723,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H55</f>
         <v>46073</v>
@@ -9779,7 +9745,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H56</f>
         <v>46074</v>
@@ -9801,7 +9767,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H57</f>
         <v>46075</v>
@@ -9823,7 +9789,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H58</f>
         <v>46076</v>
@@ -9845,7 +9811,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H59</f>
         <v>46077</v>
@@ -9867,7 +9833,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H60</f>
         <v>46078</v>
@@ -9889,7 +9855,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H61</f>
         <v>46079</v>
@@ -9911,7 +9877,7 @@
         <v>4.7399999999999998E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H62</f>
         <v>46080</v>
@@ -9933,7 +9899,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H63</f>
         <v>46081</v>
@@ -9955,7 +9921,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H64</f>
         <v>46082</v>
@@ -9977,7 +9943,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H65</f>
         <v>46083</v>
@@ -9999,7 +9965,7 @@
         <v>4.7300000000000002E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H66</f>
         <v>46084</v>
@@ -10021,7 +9987,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H67</f>
         <v>46085</v>
@@ -10043,7 +10009,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H68</f>
         <v>46086</v>
@@ -10065,7 +10031,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H69</f>
         <v>46087</v>
@@ -10087,7 +10053,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H70</f>
         <v>46088</v>
@@ -10109,7 +10075,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H71</f>
         <v>46089</v>
@@ -10131,7 +10097,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H72</f>
         <v>46090</v>
@@ -10153,7 +10119,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H73</f>
         <v>46091</v>
@@ -10175,7 +10141,7 @@
         <v>4.8500000000000001E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H74</f>
         <v>46092</v>
@@ -10197,7 +10163,7 @@
         <v>4.9099999999999998E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H75</f>
         <v>46093</v>
@@ -10219,7 +10185,7 @@
         <v>5.0099999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H76</f>
         <v>46094</v>
@@ -10241,7 +10207,7 @@
         <v>5.0700000000000002E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H77</f>
         <v>46095</v>
@@ -10263,7 +10229,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H78</f>
         <v>46096</v>
@@ -10285,7 +10251,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H79</f>
         <v>46097</v>
@@ -10307,7 +10273,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H80</f>
         <v>46098</v>
@@ -10329,7 +10295,7 @@
         <v>5.0500000000000003E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H81</f>
         <v>46099</v>
@@ -10351,7 +10317,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H82</f>
         <v>46100</v>
@@ -10373,7 +10339,7 @@
         <v>5.04E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H83</f>
         <v>46101</v>
@@ -10395,73 +10361,73 @@
         <v>5.0200000000000002E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H84</f>
         <v>46102</v>
       </c>
-      <c r="B83" s="17" t="str">
+      <c r="B83" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I84</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C83" s="47" t="str">
+        <v>4.3400000000000001E-2</v>
+      </c>
+      <c r="C83" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J84</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D83" s="47" t="str">
+        <v>4.65E-2</v>
+      </c>
+      <c r="D83" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K84</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E83" s="5" t="str">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="E83" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L84</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.1499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H85</f>
         <v>46103</v>
       </c>
-      <c r="B84" s="17" t="str">
+      <c r="B84" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I85</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C84" s="47" t="str">
+        <v>4.3400000000000001E-2</v>
+      </c>
+      <c r="C84" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J85</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D84" s="47" t="str">
+        <v>4.65E-2</v>
+      </c>
+      <c r="D84" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K85</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E84" s="5" t="str">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="E84" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L85</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.1499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H86</f>
         <v>46104</v>
       </c>
-      <c r="B85" s="17" t="str">
+      <c r="B85" s="17">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!I86</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="C85" s="47" t="str">
+        <v>4.3400000000000001E-2</v>
+      </c>
+      <c r="C85" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!J86</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="D85" s="47" t="str">
+        <v>4.65E-2</v>
+      </c>
+      <c r="D85" s="47">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!K86</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E85" s="5" t="str">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="E85" s="5">
         <f ca="1">'[1]Jumbo Bus Date to PDD'!L86</f>
-        <v xml:space="preserve"> </v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.1499999999999997E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H87</f>
         <v>46105</v>
@@ -10483,7 +10449,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H88</f>
         <v>46106</v>
@@ -10505,7 +10471,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H89</f>
         <v>46107</v>
@@ -10527,7 +10493,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H90</f>
         <v>46108</v>
@@ -10549,7 +10515,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H91</f>
         <v>46109</v>
@@ -10571,7 +10537,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H92</f>
         <v>46110</v>
@@ -10593,7 +10559,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H93</f>
         <v>46111</v>
@@ -10615,7 +10581,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H94</f>
         <v>46112</v>
@@ -10637,7 +10603,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H95</f>
         <v>46113</v>
@@ -10659,7 +10625,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H96</f>
         <v>46114</v>
@@ -10681,7 +10647,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H97</f>
         <v>46115</v>
@@ -10703,7 +10669,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H98</f>
         <v>46116</v>
@@ -10725,7 +10691,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H99</f>
         <v>46117</v>
@@ -10747,7 +10713,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H100</f>
         <v>46118</v>
@@ -10769,7 +10735,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H101</f>
         <v>46119</v>
@@ -10791,7 +10757,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H102</f>
         <v>46120</v>
@@ -10813,7 +10779,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H103</f>
         <v>46121</v>
@@ -10835,7 +10801,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H104</f>
         <v>46122</v>
@@ -10857,7 +10823,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H105</f>
         <v>46123</v>
@@ -10879,7 +10845,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H106</f>
         <v>46124</v>
@@ -10901,7 +10867,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H107</f>
         <v>46125</v>
@@ -10923,7 +10889,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H108</f>
         <v>46126</v>
@@ -10945,7 +10911,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H109</f>
         <v>46127</v>
@@ -10967,7 +10933,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H110</f>
         <v>46128</v>
@@ -10989,7 +10955,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H111</f>
         <v>46129</v>
@@ -11011,7 +10977,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H112</f>
         <v>46130</v>
@@ -11033,7 +10999,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H113</f>
         <v>46131</v>
@@ -11055,7 +11021,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H114</f>
         <v>46132</v>
@@ -11077,7 +11043,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H115</f>
         <v>46133</v>
@@ -11099,7 +11065,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H116</f>
         <v>46134</v>
@@ -11121,7 +11087,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H117</f>
         <v>46135</v>
@@ -11143,7 +11109,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H118</f>
         <v>46136</v>
@@ -11165,7 +11131,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H119</f>
         <v>46137</v>
@@ -11187,7 +11153,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H120</f>
         <v>46138</v>
@@ -11209,7 +11175,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H121</f>
         <v>46139</v>
@@ -11231,7 +11197,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H122</f>
         <v>46140</v>
@@ -11253,7 +11219,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H123</f>
         <v>46141</v>
@@ -11275,7 +11241,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H124</f>
         <v>46142</v>
@@ -11297,7 +11263,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H125</f>
         <v>46143</v>
@@ -11319,7 +11285,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H126</f>
         <v>46144</v>
@@ -11341,7 +11307,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H127</f>
         <v>46145</v>
@@ -11363,7 +11329,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H128</f>
         <v>46146</v>
@@ -11385,7 +11351,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H129</f>
         <v>46147</v>
@@ -11407,7 +11373,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H130</f>
         <v>46148</v>
@@ -11429,7 +11395,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H131</f>
         <v>46149</v>
@@ -11451,7 +11417,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H132</f>
         <v>46150</v>
@@ -11473,7 +11439,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H133</f>
         <v>46151</v>
@@ -11495,7 +11461,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H134</f>
         <v>46152</v>
@@ -11517,7 +11483,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H135</f>
         <v>46153</v>
@@ -11539,7 +11505,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H136</f>
         <v>46154</v>
@@ -11561,7 +11527,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H137</f>
         <v>46155</v>
@@ -11583,7 +11549,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H138</f>
         <v>46156</v>
@@ -11605,7 +11571,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H139</f>
         <v>46157</v>
@@ -11627,7 +11593,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H140</f>
         <v>46158</v>
@@ -11649,7 +11615,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H141</f>
         <v>46159</v>
@@ -11671,7 +11637,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H142</f>
         <v>46160</v>
@@ -11693,7 +11659,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H143</f>
         <v>46161</v>
@@ -11715,7 +11681,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H144</f>
         <v>46162</v>
@@ -11737,7 +11703,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H145</f>
         <v>46163</v>
@@ -11759,7 +11725,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H146</f>
         <v>46164</v>
@@ -11781,7 +11747,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H147</f>
         <v>46165</v>
@@ -11803,7 +11769,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H148</f>
         <v>46166</v>
@@ -11825,7 +11791,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H149</f>
         <v>46167</v>
@@ -11847,7 +11813,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H150</f>
         <v>46168</v>
@@ -11869,7 +11835,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H151</f>
         <v>46169</v>
@@ -11891,7 +11857,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H152</f>
         <v>46170</v>
@@ -11913,7 +11879,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H153</f>
         <v>46171</v>
@@ -11935,7 +11901,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H154</f>
         <v>46172</v>
@@ -11957,7 +11923,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H155</f>
         <v>46173</v>
@@ -11979,7 +11945,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H156</f>
         <v>46174</v>
@@ -12001,7 +11967,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H157</f>
         <v>46175</v>
@@ -12023,7 +11989,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H158</f>
         <v>46176</v>
@@ -12045,7 +12011,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H159</f>
         <v>46177</v>
@@ -12067,7 +12033,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H160</f>
         <v>46178</v>
@@ -12089,7 +12055,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H161</f>
         <v>46179</v>
@@ -12111,7 +12077,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H162</f>
         <v>46180</v>
@@ -12133,7 +12099,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H163</f>
         <v>46181</v>
@@ -12155,7 +12121,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H164</f>
         <v>46182</v>
@@ -12177,7 +12143,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H165</f>
         <v>46183</v>
@@ -12199,7 +12165,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H166</f>
         <v>46184</v>
@@ -12221,7 +12187,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H167</f>
         <v>46185</v>
@@ -12243,7 +12209,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H168</f>
         <v>46186</v>
@@ -12265,7 +12231,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H169</f>
         <v>46187</v>
@@ -12287,7 +12253,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H170</f>
         <v>46188</v>
@@ -12309,7 +12275,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H171</f>
         <v>46189</v>
@@ -12331,7 +12297,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H172</f>
         <v>46190</v>
@@ -12353,7 +12319,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H173</f>
         <v>46191</v>
@@ -12375,7 +12341,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H174</f>
         <v>46192</v>
@@ -12397,7 +12363,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H175</f>
         <v>46193</v>
@@ -12419,7 +12385,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H176</f>
         <v>46194</v>
@@ -12441,7 +12407,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H177</f>
         <v>46195</v>
@@ -12463,7 +12429,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H178</f>
         <v>46196</v>
@@ -12485,7 +12451,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H179</f>
         <v>46197</v>
@@ -12507,7 +12473,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H180</f>
         <v>46198</v>
@@ -12529,7 +12495,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H181</f>
         <v>46199</v>
@@ -12551,7 +12517,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H182</f>
         <v>46200</v>
@@ -12573,7 +12539,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H183</f>
         <v>46201</v>
@@ -12595,7 +12561,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H184</f>
         <v>46202</v>
@@ -12617,7 +12583,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H185</f>
         <v>46203</v>
@@ -12639,7 +12605,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H186</f>
         <v>46204</v>
@@ -12661,7 +12627,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H187</f>
         <v>46205</v>
@@ -12683,7 +12649,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H188</f>
         <v>46206</v>
@@ -12705,7 +12671,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H189</f>
         <v>46207</v>
@@ -12727,7 +12693,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H190</f>
         <v>46208</v>
@@ -12749,7 +12715,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H191</f>
         <v>46209</v>
@@ -12771,7 +12737,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H192</f>
         <v>46210</v>
@@ -12793,7 +12759,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H193</f>
         <v>46211</v>
@@ -12815,7 +12781,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H194</f>
         <v>46212</v>
@@ -12837,7 +12803,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H195</f>
         <v>46213</v>
@@ -12859,7 +12825,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H196</f>
         <v>46214</v>
@@ -12881,7 +12847,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H197</f>
         <v>46215</v>
@@ -12903,7 +12869,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H198</f>
         <v>46216</v>
@@ -12925,7 +12891,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H199</f>
         <v>46217</v>
@@ -12947,7 +12913,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H200</f>
         <v>46218</v>
@@ -12969,7 +12935,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H201</f>
         <v>46219</v>
@@ -12991,7 +12957,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H202</f>
         <v>46220</v>
@@ -13013,7 +12979,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H203</f>
         <v>46221</v>
@@ -13035,7 +13001,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H204</f>
         <v>46222</v>
@@ -13057,7 +13023,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H205</f>
         <v>46223</v>
@@ -13079,7 +13045,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H206</f>
         <v>46224</v>
@@ -13101,7 +13067,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H207</f>
         <v>46225</v>
@@ -13123,7 +13089,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H208</f>
         <v>46226</v>
@@ -13145,7 +13111,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H209</f>
         <v>46227</v>
@@ -13167,7 +13133,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H210</f>
         <v>46228</v>
@@ -13189,7 +13155,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H211</f>
         <v>46229</v>
@@ -13211,7 +13177,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H212</f>
         <v>46230</v>
@@ -13233,7 +13199,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H213</f>
         <v>46231</v>
@@ -13255,7 +13221,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H214</f>
         <v>46232</v>
@@ -13277,7 +13243,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H215</f>
         <v>46233</v>
@@ -13299,7 +13265,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H216</f>
         <v>46234</v>
@@ -13321,7 +13287,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H217</f>
         <v>46235</v>
@@ -13343,7 +13309,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H218</f>
         <v>46236</v>
@@ -13365,7 +13331,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H219</f>
         <v>46237</v>
@@ -13387,7 +13353,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H220</f>
         <v>46238</v>
@@ -13409,7 +13375,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H221</f>
         <v>46239</v>
@@ -13431,7 +13397,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H222</f>
         <v>46240</v>
@@ -13453,7 +13419,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H223</f>
         <v>46241</v>
@@ -13475,7 +13441,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H224</f>
         <v>46242</v>
@@ -13497,7 +13463,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H225</f>
         <v>46243</v>
@@ -13519,7 +13485,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H226</f>
         <v>46244</v>
@@ -13541,7 +13507,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H227</f>
         <v>46245</v>
@@ -13563,7 +13529,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H228</f>
         <v>46246</v>
@@ -13585,7 +13551,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H229</f>
         <v>46247</v>
@@ -13607,7 +13573,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H230</f>
         <v>46248</v>
@@ -13629,7 +13595,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H231</f>
         <v>46249</v>
@@ -13651,7 +13617,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H232</f>
         <v>46250</v>
@@ -13673,7 +13639,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H233</f>
         <v>46251</v>
@@ -13695,7 +13661,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H234</f>
         <v>46252</v>
@@ -13717,7 +13683,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H235</f>
         <v>46253</v>
@@ -13739,7 +13705,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H236</f>
         <v>46254</v>
@@ -13761,7 +13727,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H237</f>
         <v>46255</v>
@@ -13783,7 +13749,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H238</f>
         <v>46256</v>
@@ -13805,7 +13771,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H239</f>
         <v>46257</v>
@@ -13827,7 +13793,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H240</f>
         <v>46258</v>
@@ -13849,7 +13815,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H241</f>
         <v>46259</v>
@@ -13871,7 +13837,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="15">
         <f>'[1]Jumbo Bus Date to PDD'!H242</f>
         <v>46260</v>
@@ -13893,7 +13859,7 @@
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    